<commit_message>
Prepare Basel credit capital engine for publication
</commit_message>
<xml_diff>
--- a/outputs/demo/Basel_Credit_Capital_Report.xlsx
+++ b/outputs/demo/Basel_Credit_Capital_Report.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Executive_Summary" sheetId="1" r:id="R3f41d6e6a8e94bec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Portfolio_Profile" sheetId="2" r:id="Ra4f0d342f0ca41b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_SA_RWA" sheetId="3" r:id="R7c37d60752eb45bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_IRB_RWA" sheetId="4" r:id="Rfe876b8dafb245ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_SA_vs_IRB" sheetId="5" r:id="Ree3c5c4f0d1e4059"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Concentration" sheetId="6" r:id="R7ec7de8b164048ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_RWA_Bridge" sheetId="7" r:id="R4a1869b70a7c4bda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Stress_Test" sheetId="8" r:id="Rdb63ea1b9f504d05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Capital_Adequacy" sheetId="9" r:id="Rf5c0e7d22ab2454c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Reconciliation" sheetId="10" r:id="Re83e9d0b114c4b6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Methodology" sheetId="11" r:id="R809e36bffe274b52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Executive_Summary" sheetId="1" r:id="R3026e59171dc4de5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Portfolio_Profile" sheetId="2" r:id="R5f984c9416c14383"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_SA_RWA" sheetId="3" r:id="R3e09b7e527d34a9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_IRB_RWA" sheetId="4" r:id="R95500ed8de7b4f0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_SA_vs_IRB" sheetId="5" r:id="R2ae4f0afefd84f14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Concentration" sheetId="6" r:id="R159901475cf94171"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_RWA_Bridge" sheetId="7" r:id="Rfcaaf4e595f64a63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Stress_Test" sheetId="8" r:id="R267a9dcd9d9f40d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Capital_Adequacy" sheetId="9" r:id="R8a30817c2e7949dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Reconciliation" sheetId="10" r:id="Rfbc7bb5b02ea4f22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Methodology" sheetId="11" r:id="R9db7f455a9814ec9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23,15 +23,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.0;[Red](#,##0.0);-"/>
     <x:numFmt numFmtId="202" formatCode="0.0%;[Red](0.0%);-"/>
     <x:numFmt numFmtId="203" formatCode="0.0000"/>
     <x:numFmt numFmtId="204" formatCode="0.00x"/>
     <x:numFmt numFmtId="205" formatCode="0.0000%"/>
+    <x:numFmt numFmtId="206" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="20">
+  <x:fonts count="22">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -142,8 +143,19 @@
       <x:color rgb="FF1E8449"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -178,6 +190,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF2A9D8F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF247FB3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B3F56"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -240,7 +267,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="173">
+  <x:cellXfs count="185">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -678,6 +705,36 @@
     <x:xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="206" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -689,7 +746,7 @@
         <x:color rgb="FFC0392B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFADBD8"/>
         </x:patternFill>
       </x:fill>
@@ -700,7 +757,7 @@
         <x:color rgb="FF1E8449"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD5F5E3"/>
         </x:patternFill>
       </x:fill>
@@ -711,7 +768,7 @@
         <x:color rgb="FF1E8449"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD5F5E3"/>
         </x:patternFill>
       </x:fill>
@@ -722,7 +779,7 @@
         <x:color rgb="FFC0392B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFADBD8"/>
         </x:patternFill>
       </x:fill>
@@ -1073,7 +1130,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:t>SA versus IRB Credit RWA by class (INR crore)</a:t>
+              <a:t>Credit RWA intensity by class</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1088,11 +1145,11 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Sa Rwa (INR crore)</c:v>
+            <c:v>SA RWA / EAD</c:v>
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'05_SA_vs_IRB'!$A$5:$A$14</c:f>
+              <c:f>'05_SA_vs_IRB'!$H$21:$H$30</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -1100,9 +1157,9 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'05_SA_vs_IRB'!$B$5:$B$14</c:f>
+              <c:f>'05_SA_vs_IRB'!$I$21:$I$30</c:f>
               <c:numCache>
-                <c:formatCode>#,##0.0;[Red](#,##0.0);-</c:formatCode>
+                <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
               </c:numCache>
             </c:numRef>
@@ -1112,11 +1169,11 @@
           <c:idx val="1"/>
           <c:order val="1"/>
           <c:tx>
-            <c:v>Irb Rwa (INR crore)</c:v>
+            <c:v>IRB RWA / EAD</c:v>
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'05_SA_vs_IRB'!$A$5:$A$14</c:f>
+              <c:f>'05_SA_vs_IRB'!$H$21:$H$30</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -1124,9 +1181,9 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'05_SA_vs_IRB'!$C$5:$C$14</c:f>
+              <c:f>'05_SA_vs_IRB'!$J$21:$J$30</c:f>
               <c:numCache>
-                <c:formatCode>#,##0.0;[Red](#,##0.0);-</c:formatCode>
+                <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="0"/>
               </c:numCache>
             </c:numRef>
@@ -1175,7 +1232,7 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="#,##0"/>
+        <c:numFmt formatCode="0%"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:crossAx val="48650112"/>
@@ -1230,7 +1287,7 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>'07_RWA_Bridge'!$A$6:$A$12</c:f>
+              <c:f>'07_RWA_Bridge'!$A$6:$A$13</c:f>
               <c:strCache>
                 <c:ptCount val="0"/>
               </c:strCache>
@@ -1238,7 +1295,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'07_RWA_Bridge'!$B$6:$B$12</c:f>
+              <c:f>'07_RWA_Bridge'!$B$6:$B$13</c:f>
               <c:numCache>
                 <c:formatCode>#,##0.0;[Red](#,##0.0);-</c:formatCode>
                 <c:ptCount val="0"/>
@@ -1555,7 +1612,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R503b438347614958"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfc2c8e125ed44c57"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1585,7 +1642,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re1a8a24b82c348d7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd8f5c5d8cf844870"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1620,7 +1677,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfb7ed5a91ccc4b93"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0afdd98462264ab9"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1655,7 +1712,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R156fb2cecab949e5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5d045229ada94570"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1690,7 +1747,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R507cdf740a9d4ace"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R394e7a2c98354b79"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1725,7 +1782,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3d64c511741b4017"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ref63cac383734f17"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1760,7 +1817,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6f54926efd324ee9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R813af828a8a14ec8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2245,7 +2302,7 @@
       </x:c>
       <x:c r="B6" s="114" t="n">
         <x:f>'02_Portfolio_Profile'!B9</x:f>
-        <x:v>702887.8163117705</x:v>
+        <x:v>700735.4648341014</x:v>
       </x:c>
       <x:c r="C6" s="108"/>
       <x:c r="D6" s="115" t="str">
@@ -2266,7 +2323,7 @@
       </x:c>
       <x:c r="B7" s="114" t="n">
         <x:f>'02_Portfolio_Profile'!B10</x:f>
-        <x:v>406207.69049290236</x:v>
+        <x:v>405323.35943071585</x:v>
       </x:c>
       <x:c r="C7" s="108"/>
       <x:c r="D7" s="115"/>
@@ -2285,7 +2342,7 @@
       </x:c>
       <x:c r="B8" s="114" t="n">
         <x:f>'02_Portfolio_Profile'!B11</x:f>
-        <x:v>728676.4076818405</x:v>
+        <x:v>583349.2328979744</x:v>
       </x:c>
       <x:c r="C8" s="108"/>
       <x:c r="D8" s="115"/>
@@ -2304,7 +2361,7 @@
       </x:c>
       <x:c r="B9" s="114" t="n">
         <x:f>'08_Stress_Test'!F5</x:f>
-        <x:v>753676.4076818405</x:v>
+        <x:v>608349.2328979744</x:v>
       </x:c>
       <x:c r="C9" s="108"/>
       <x:c r="D9" s="115"/>
@@ -2323,7 +2380,7 @@
       </x:c>
       <x:c r="B10" s="116" t="n">
         <x:f>'09_Capital_Adequacy'!E5</x:f>
-        <x:v>0.0862439096</x:v>
+        <x:v>0.1068465225</x:v>
       </x:c>
       <x:c r="C10" s="108"/>
       <x:c r="D10" s="115"/>
@@ -2342,7 +2399,7 @@
       </x:c>
       <x:c r="B11" s="116" t="n">
         <x:f>'09_Capital_Adequacy'!E8</x:f>
-        <x:v>0.055948805</x:v>
+        <x:v>0.0705336941</x:v>
       </x:c>
       <x:c r="C11" s="108"/>
       <x:c r="D11" s="115"/>
@@ -2361,7 +2418,7 @@
       </x:c>
       <x:c r="B12" s="118" t="n">
         <x:f>'09_Capital_Adequacy'!E11</x:f>
-        <x:v>0.0314148507</x:v>
+        <x:v>0.0401329226</x:v>
       </x:c>
       <x:c r="C12" s="108"/>
       <x:c r="D12" s="115"/>
@@ -2444,11 +2501,11 @@
       </x:c>
       <x:c r="B17" s="120" t="n">
         <x:f>'08_Stress_Test'!F5</x:f>
-        <x:v>753676.4076818405</x:v>
+        <x:v>608349.2328979744</x:v>
       </x:c>
       <x:c r="C17" s="121" t="n">
         <x:f>'09_Capital_Adequacy'!E5</x:f>
-        <x:v>0.0862439096</x:v>
+        <x:v>0.1068465225</x:v>
       </x:c>
       <x:c r="D17" s="108"/>
       <x:c r="E17" s="108"/>
@@ -2466,11 +2523,11 @@
       </x:c>
       <x:c r="B18" s="120" t="n">
         <x:f>'08_Stress_Test'!F6</x:f>
-        <x:v>1001102.9494243957</x:v>
+        <x:v>794539.1397440645</x:v>
       </x:c>
       <x:c r="C18" s="121" t="n">
         <x:f>'09_Capital_Adequacy'!E8</x:f>
-        <x:v>0.055948805</x:v>
+        <x:v>0.0705336941</x:v>
       </x:c>
       <x:c r="D18" s="108"/>
       <x:c r="E18" s="108"/>
@@ -2488,11 +2545,11 @@
       </x:c>
       <x:c r="B19" s="120" t="n">
         <x:f>'08_Stress_Test'!F7</x:f>
-        <x:v>1292671.0865599755</x:v>
+        <x:v>1013975.0971355619</x:v>
       </x:c>
       <x:c r="C19" s="121" t="n">
         <x:f>'09_Capital_Adequacy'!E11</x:f>
-        <x:v>0.0314148507</x:v>
+        <x:v>0.0401329226</x:v>
       </x:c>
       <x:c r="D19" s="108"/>
       <x:c r="E19" s="108"/>
@@ -2514,7 +2571,7 @@
     <x:mergeCell ref="A15:H15"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c68eda2af6b4314"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62e27a5c3ebd458d"/>
 </x:worksheet>
 </file>
 
@@ -2660,15 +2717,15 @@
       </x:c>
       <x:c r="B6" s="162" t="n">
         <x:f>SUM('03_SA_RWA'!B5:B14)</x:f>
-        <x:v>702887.8163117705</x:v>
+        <x:v>700735.4648341016</x:v>
       </x:c>
       <x:c r="C6" s="162" t="n">
         <x:f>'02_Portfolio_Profile'!B9</x:f>
-        <x:v>702887.8163117705</x:v>
+        <x:v>700735.4648341014</x:v>
       </x:c>
       <x:c r="D6" s="163" t="n">
         <x:f>B6-C6</x:f>
-        <x:v>0</x:v>
+        <x:v>2.3283064365386963e-10</x:v>
       </x:c>
       <x:c r="E6" s="163" t="n">
         <x:v>0.0001</x:v>
@@ -2698,11 +2755,11 @@
       </x:c>
       <x:c r="B7" s="162" t="n">
         <x:f>SUM('03_SA_RWA'!D5:D14)</x:f>
-        <x:v>406207.6904929024</x:v>
+        <x:v>405323.3594307159</x:v>
       </x:c>
       <x:c r="C7" s="162" t="n">
         <x:f>'02_Portfolio_Profile'!B10</x:f>
-        <x:v>406207.69049290236</x:v>
+        <x:v>405323.35943071585</x:v>
       </x:c>
       <x:c r="D7" s="163" t="n">
         <x:f>B7-C7</x:f>
@@ -2736,15 +2793,15 @@
       </x:c>
       <x:c r="B8" s="162" t="n">
         <x:f>SUM('04_IRB_RWA'!F5:F14)</x:f>
-        <x:v>728676.4076818406</x:v>
+        <x:v>583349.2328979743</x:v>
       </x:c>
       <x:c r="C8" s="162" t="n">
         <x:f>'02_Portfolio_Profile'!B11</x:f>
-        <x:v>728676.4076818405</x:v>
+        <x:v>583349.2328979744</x:v>
       </x:c>
       <x:c r="D8" s="163" t="n">
         <x:f>B8-C8</x:f>
-        <x:v>1.1641532182693481e-10</x:v>
+        <x:v>-1.1641532182693481e-10</x:v>
       </x:c>
       <x:c r="E8" s="163" t="n">
         <x:v>0.0001</x:v>
@@ -2762,7 +2819,7 @@
         <x:v>Gross balance</x:v>
       </x:c>
       <x:c r="K8" s="132" t="n">
-        <x:v>558645.0087404712</x:v>
+        <x:v>558161.9862245091</x:v>
       </x:c>
       <x:c r="L8" s="130" t="str">
         <x:v>PASS</x:v>
@@ -2773,16 +2830,16 @@
         <x:v>Prior RWA plus drivers equals current RWA</x:v>
       </x:c>
       <x:c r="B9" s="162" t="n">
-        <x:f>'07_RWA_Bridge'!B5+SUM('07_RWA_Bridge'!B6:B12)</x:f>
-        <x:v>728676.4076818405</x:v>
+        <x:f>'07_RWA_Bridge'!B5+SUM('07_RWA_Bridge'!B6:B13)</x:f>
+        <x:v>583349.2328979746</x:v>
       </x:c>
       <x:c r="C9" s="162" t="n">
-        <x:f>'07_RWA_Bridge'!B13</x:f>
-        <x:v>728676.4076818405</x:v>
+        <x:f>'07_RWA_Bridge'!B14</x:f>
+        <x:v>583349.2328979744</x:v>
       </x:c>
       <x:c r="D9" s="163" t="n">
         <x:f>B9-C9</x:f>
-        <x:v>0</x:v>
+        <x:v>1.1641532182693481e-10</x:v>
       </x:c>
       <x:c r="E9" s="163" t="n">
         <x:v>0.0001</x:v>
@@ -2800,7 +2857,7 @@
         <x:v>Undrawn amount</x:v>
       </x:c>
       <x:c r="K9" s="137" t="n">
-        <x:v>352270.5553538803</x:v>
+        <x:v>348131.18875714944</x:v>
       </x:c>
       <x:c r="L9" s="135" t="str">
         <x:v>PASS</x:v>
@@ -2812,11 +2869,11 @@
       </x:c>
       <x:c r="B10" s="162" t="n">
         <x:f>'09_Capital_Adequacy'!D5</x:f>
-        <x:v>753676.4076818405</x:v>
+        <x:v>608349.2328979744</x:v>
       </x:c>
       <x:c r="C10" s="162" t="n">
         <x:f>'08_Stress_Test'!F5</x:f>
-        <x:v>753676.4076818405</x:v>
+        <x:v>608349.2328979744</x:v>
       </x:c>
       <x:c r="D10" s="163" t="n">
         <x:f>B10-C10</x:f>
@@ -2844,15 +2901,15 @@
       </x:c>
       <x:c r="B11" s="166" t="n">
         <x:f>'09_Capital_Adequacy'!E5</x:f>
-        <x:v>0.0862439096</x:v>
+        <x:v>0.1068465225</x:v>
       </x:c>
       <x:c r="C11" s="166" t="n">
         <x:f>'09_Capital_Adequacy'!C5/'09_Capital_Adequacy'!D5</x:f>
-        <x:v>0.0862439096374625</x:v>
+        <x:v>0.10684652249886387</x:v>
       </x:c>
       <x:c r="D11" s="166" t="n">
         <x:f>B11-C11</x:f>
-        <x:v>-3.74625053201072e-11</x:v>
+        <x:v>1.1361328544623461e-12</x:v>
       </x:c>
       <x:c r="E11" s="166" t="n">
         <x:v>1e-7</x:v>
@@ -3329,7 +3386,7 @@
         <x:v>RBC90</x:v>
       </x:c>
       <x:c r="B20" s="170" t="str">
-        <x:v>Output-floor transition</x:v>
+        <x:v>Output-floor transitional calibration</x:v>
       </x:c>
       <x:c r="C20" s="170" t="str">
         <x:v>https://www.bis.org/basel_framework/chapter/RBC/90.htm</x:v>
@@ -3351,13 +3408,13 @@
         <x:v>CRE20</x:v>
       </x:c>
       <x:c r="B21" s="170" t="str">
-        <x:v>Standardised Approach exposures</x:v>
+        <x:v>SA classes, retail/SME eligibility and CCFs</x:v>
       </x:c>
       <x:c r="C21" s="170" t="str">
-        <x:v>https://www.bis.org/basel_framework/chapter/CRE/20.htm</x:v>
+        <x:v>https://www.bis.org/committees/bcbs/basel-framework/standard/cre/20/inforce/2023-01-01/published/2020-11-26</x:v>
       </x:c>
       <x:c r="D21" s="170" t="str">
-        <x:v>Accessed 2026-08-22</x:v>
+        <x:v>Accessed 2026-08-31; 20.47, 20.65–68, 20.95–100</x:v>
       </x:c>
       <x:c r="E21" s="108"/>
       <x:c r="F21" s="108"/>
@@ -3414,13 +3471,13 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="170" t="str">
-        <x:v>CRE31</x:v>
+        <x:v>CRE30</x:v>
       </x:c>
       <x:c r="B24" s="170" t="str">
-        <x:v>IRB risk-weight functions</x:v>
+        <x:v>IRB classes and restrictions</x:v>
       </x:c>
       <x:c r="C24" s="170" t="str">
-        <x:v>https://www.bis.org/basel_framework/chapter/CRE/31.htm</x:v>
+        <x:v>https://www.bis.org/basel_framework/chapter/CRE/30.htm</x:v>
       </x:c>
       <x:c r="D24" s="170" t="str">
         <x:v>Accessed 2026-08-22</x:v>
@@ -3436,13 +3493,13 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="170" t="str">
-        <x:v>DIS40</x:v>
+        <x:v>CRE31</x:v>
       </x:c>
       <x:c r="B25" s="170" t="str">
-        <x:v>Credit-risk disclosure concepts</x:v>
+        <x:v>IRB risk-weight functions</x:v>
       </x:c>
       <x:c r="C25" s="170" t="str">
-        <x:v>https://www.bis.org/basel_framework/chapter/DIS/40.htm</x:v>
+        <x:v>https://www.bis.org/basel_framework/chapter/CRE/31.htm</x:v>
       </x:c>
       <x:c r="D25" s="170" t="str">
         <x:v>Accessed 2026-08-22</x:v>
@@ -3458,16 +3515,16 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="170" t="str">
-        <x:v>MAR20</x:v>
+        <x:v>CRE32</x:v>
       </x:c>
       <x:c r="B26" s="170" t="str">
-        <x:v>Market-risk capital and RWA</x:v>
+        <x:v>Foundation LGD, floors, EAD and maturity</x:v>
       </x:c>
       <x:c r="C26" s="170" t="str">
-        <x:v>https://www.bis.org/basel_framework/chapter/MAR/20.htm</x:v>
+        <x:v>https://www.bis.org/committees/bcbs/basel-framework/standard/cre/32/inforce/2023-01-01/published/2020-03-27</x:v>
       </x:c>
       <x:c r="D26" s="170" t="str">
-        <x:v>Accessed 2026-08-23</x:v>
+        <x:v>Accessed 2026-08-31; 32.6, 32.10–11, 32.16, 32.36, 32.44–48, 32.58</x:v>
       </x:c>
       <x:c r="E26" s="108"/>
       <x:c r="F26" s="108"/>
@@ -3480,16 +3537,16 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="170" t="str">
-        <x:v>OPE25</x:v>
+        <x:v>CRE36</x:v>
       </x:c>
       <x:c r="B27" s="170" t="str">
-        <x:v>Operational-risk Standardised Approach</x:v>
+        <x:v>IRB estimation and stress requirements</x:v>
       </x:c>
       <x:c r="C27" s="170" t="str">
-        <x:v>https://www.bis.org/basel_framework/chapter/OPE/25.htm</x:v>
+        <x:v>https://www.bis.org/basel_framework/chapter/CRE/36.htm</x:v>
       </x:c>
       <x:c r="D27" s="170" t="str">
-        <x:v>Accessed 2026-08-23</x:v>
+        <x:v>Accessed 2026-08-22</x:v>
       </x:c>
       <x:c r="E27" s="108"/>
       <x:c r="F27" s="108"/>
@@ -3502,13 +3559,13 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="170" t="str">
-        <x:v>CRE36</x:v>
+        <x:v>MAR20</x:v>
       </x:c>
       <x:c r="B28" s="170" t="str">
-        <x:v>IRB estimation and stress requirements</x:v>
+        <x:v>Market-risk capital and RWA</x:v>
       </x:c>
       <x:c r="C28" s="170" t="str">
-        <x:v>https://www.bis.org/basel_framework/chapter/CRE/36.htm</x:v>
+        <x:v>https://www.bis.org/basel_framework/chapter/MAR/20.htm</x:v>
       </x:c>
       <x:c r="D28" s="170" t="str">
         <x:v>Accessed 2026-08-23</x:v>
@@ -3524,13 +3581,13 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="171" t="str">
-        <x:v>BCBS Stress</x:v>
+        <x:v>OPE10</x:v>
       </x:c>
       <x:c r="B29" s="171" t="str">
-        <x:v>Stress-testing principles</x:v>
+        <x:v>Operational-risk definitions</x:v>
       </x:c>
       <x:c r="C29" s="171" t="str">
-        <x:v>https://www.bis.org/bcbs/publ/d450.htm</x:v>
+        <x:v>https://www.bis.org/basel_framework/chapter/OPE/10.htm</x:v>
       </x:c>
       <x:c r="D29" s="171" t="str">
         <x:v>Accessed 2026-08-23</x:v>
@@ -3545,10 +3602,18 @@
       <x:c r="L29" s="108"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="108"/>
-      <x:c r="B30" s="108"/>
-      <x:c r="C30" s="108"/>
-      <x:c r="D30" s="108"/>
+      <x:c r="A30" s="176" t="str">
+        <x:v>OPE25</x:v>
+      </x:c>
+      <x:c r="B30" s="176" t="str">
+        <x:v>Operational-risk Standardised Approach</x:v>
+      </x:c>
+      <x:c r="C30" s="176" t="str">
+        <x:v>https://www.bis.org/basel_framework/chapter/OPE/25.htm</x:v>
+      </x:c>
+      <x:c r="D30" s="176" t="str">
+        <x:v>Accessed 2026-08-23</x:v>
+      </x:c>
       <x:c r="E30" s="108"/>
       <x:c r="F30" s="108"/>
       <x:c r="G30" s="108"/>
@@ -3559,10 +3624,18 @@
       <x:c r="L30" s="108"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="108"/>
-      <x:c r="B31" s="108"/>
-      <x:c r="C31" s="108"/>
-      <x:c r="D31" s="108"/>
+      <x:c r="A31" s="176" t="str">
+        <x:v>BCBS Stress</x:v>
+      </x:c>
+      <x:c r="B31" s="176" t="str">
+        <x:v>Stress-testing principles</x:v>
+      </x:c>
+      <x:c r="C31" s="176" t="str">
+        <x:v>https://www.bis.org/bcbs/publ/d450.htm</x:v>
+      </x:c>
+      <x:c r="D31" s="176" t="str">
+        <x:v>Accessed 2026-08-23</x:v>
+      </x:c>
       <x:c r="E31" s="108"/>
       <x:c r="F31" s="108"/>
       <x:c r="G31" s="108"/>
@@ -3573,12 +3646,18 @@
       <x:c r="L31" s="108"/>
     </x:row>
     <x:row r="32" ht="22" customHeight="1">
-      <x:c r="A32" s="109" t="str">
-        <x:v>Key limitations</x:v>
-      </x:c>
-      <x:c r="B32" s="109"/>
-      <x:c r="C32" s="109"/>
-      <x:c r="D32" s="108"/>
+      <x:c r="A32" s="180" t="str">
+        <x:v>DIS40</x:v>
+      </x:c>
+      <x:c r="B32" s="180" t="str">
+        <x:v>Credit-risk disclosure concepts</x:v>
+      </x:c>
+      <x:c r="C32" s="180" t="str">
+        <x:v>https://www.bis.org/basel_framework/chapter/DIS/40.htm</x:v>
+      </x:c>
+      <x:c r="D32" s="181" t="str">
+        <x:v>Accessed 2026-08-22</x:v>
+      </x:c>
       <x:c r="E32" s="108"/>
       <x:c r="F32" s="108"/>
       <x:c r="G32" s="108"/>
@@ -3589,9 +3668,7 @@
       <x:c r="L32" s="108"/>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
-      <x:c r="A33" s="172" t="str">
-        <x:v>All data are synthetic.</x:v>
-      </x:c>
+      <x:c r="A33" s="172"/>
       <x:c r="B33" s="172"/>
       <x:c r="C33" s="172"/>
       <x:c r="D33" s="108"/>
@@ -3605,11 +3682,15 @@
       <x:c r="L33" s="108"/>
     </x:row>
     <x:row r="34" ht="28" customHeight="1">
-      <x:c r="A34" s="172" t="str">
-        <x:v>The IRB layer demonstrates formula mechanics and does not imply supervisory approval.</x:v>
-      </x:c>
-      <x:c r="B34" s="172"/>
-      <x:c r="C34" s="172"/>
+      <x:c r="A34" s="183" t="str">
+        <x:v>Key limitations</x:v>
+      </x:c>
+      <x:c r="B34" s="183" t="str">
+        <x:v>Key limitations</x:v>
+      </x:c>
+      <x:c r="C34" s="183" t="str">
+        <x:v>Key limitations</x:v>
+      </x:c>
       <x:c r="D34" s="108"/>
       <x:c r="E34" s="108"/>
       <x:c r="F34" s="108"/>
@@ -3622,7 +3703,7 @@
     </x:row>
     <x:row r="35" ht="28" customHeight="1">
       <x:c r="A35" s="172" t="str">
-        <x:v>National implementation choices and transition schedules can differ.</x:v>
+        <x:v>All data and model parameters are synthetic.</x:v>
       </x:c>
       <x:c r="B35" s="172"/>
       <x:c r="C35" s="172"/>
@@ -3638,7 +3719,7 @@
     </x:row>
     <x:row r="36" ht="28" customHeight="1">
       <x:c r="A36" s="172" t="str">
-        <x:v>Market and Operational RWA are synthetic configured inputs; their calculation routes are shown above.</x:v>
+        <x:v>IRB mixes foundation and own-estimate routes and does not imply supervisory approval.</x:v>
       </x:c>
       <x:c r="B36" s="172"/>
       <x:c r="C36" s="172"/>
@@ -3654,7 +3735,7 @@
     </x:row>
     <x:row r="37" ht="28" customHeight="1">
       <x:c r="A37" s="172" t="str">
-        <x:v>CCR, CVA, securitisation, FRTB and full market- and operational-risk engines are outside scope.</x:v>
+        <x:v>SA guarantee recognition is simplified; guarantees are not recognised in the project IRB calculation.</x:v>
       </x:c>
       <x:c r="B37" s="172"/>
       <x:c r="C37" s="172"/>
@@ -3668,17 +3749,32 @@
       <x:c r="K37" s="108"/>
       <x:c r="L37" s="108"/>
     </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="184" t="str">
+        <x:v>Market and Operational RWA are synthetic configured inputs; their calculation routes are shown above.</x:v>
+      </x:c>
+      <x:c r="B38" s="184"/>
+      <x:c r="C38" s="184"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="184" t="str">
+        <x:v>CCR, CVA, securitisation, FRTB and full defaulted-exposure treatments are outside scope.</x:v>
+      </x:c>
+      <x:c r="B39" s="184"/>
+      <x:c r="C39" s="184"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:L1"/>
     <x:mergeCell ref="A2:L2"/>
     <x:mergeCell ref="A17:D17"/>
-    <x:mergeCell ref="A32:C32"/>
     <x:mergeCell ref="A33:C33"/>
     <x:mergeCell ref="A34:C34"/>
     <x:mergeCell ref="A35:C35"/>
     <x:mergeCell ref="A36:C36"/>
     <x:mergeCell ref="A37:C37"/>
+    <x:mergeCell ref="A38:C38"/>
+    <x:mergeCell ref="A39:C39"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3822,31 +3918,31 @@
         <x:v>Financial Services</x:v>
       </x:c>
       <x:c r="E6" s="127" t="n">
-        <x:v>147529.2334179946</x:v>
+        <x:v>139931.41796662714</x:v>
       </x:c>
       <x:c r="F6" s="127" t="n">
-        <x:v>76355.09254906393</x:v>
+        <x:v>68578.03193918924</x:v>
       </x:c>
       <x:c r="G6" s="127" t="n">
-        <x:v>132649.33399403136</x:v>
+        <x:v>88125.88688061282</x:v>
       </x:c>
       <x:c r="H6" s="126" t="n">
-        <x:v>1802</x:v>
+        <x:v>1771</x:v>
       </x:c>
       <x:c r="I6" s="128" t="n">
-        <x:v>0.209890156</x:v>
+        <x:v>0.1996922162</x:v>
       </x:c>
       <x:c r="J6" s="128" t="n">
-        <x:v>0.1820414832</x:v>
+        <x:v>0.1510688313</x:v>
       </x:c>
       <x:c r="K6" s="129" t="n">
-        <x:v>0.0440538776</x:v>
+        <x:v>0.0398769812</x:v>
       </x:c>
       <x:c r="L6" s="128" t="n">
-        <x:v>0.0135690885</x:v>
+        <x:v>0.0160565743</x:v>
       </x:c>
       <x:c r="M6" s="128" t="n">
-        <x:v>0.797737716</x:v>
+        <x:v>0.5305001493</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -3861,28 +3957,28 @@
         <x:v>Government</x:v>
       </x:c>
       <x:c r="E7" s="132" t="n">
-        <x:v>136416.9025098093</x:v>
+        <x:v>139386.41947664847</x:v>
       </x:c>
       <x:c r="F7" s="132" t="n">
-        <x:v>21593.660292094177</x:v>
+        <x:v>19020.99985192112</x:v>
       </x:c>
       <x:c r="G7" s="132" t="n">
-        <x:v>28665.82682924301</x:v>
+        <x:v>25475.185787076643</x:v>
       </x:c>
       <x:c r="H7" s="131" t="n">
         <x:v>750</x:v>
       </x:c>
       <x:c r="I7" s="133" t="n">
-        <x:v>0.194080619</x:v>
+        <x:v>0.1989144641</x:v>
       </x:c>
       <x:c r="J7" s="133" t="n">
-        <x:v>0.0393395841</x:v>
+        <x:v>0.0436705568</x:v>
       </x:c>
       <x:c r="K7" s="134" t="n">
-        <x:v>0.0376672867</x:v>
+        <x:v>0.039566964</x:v>
       </x:c>
       <x:c r="L7" s="133" t="n">
-        <x:v>0.0017969369</x:v>
+        <x:v>0.0003817235</x:v>
       </x:c>
       <x:c r="M7" s="133" t="n">
         <x:v>0.7621587156</x:v>
@@ -3893,38 +3989,38 @@
         <x:v>Gross exposure</x:v>
       </x:c>
       <x:c r="B8" s="132" t="n">
-        <x:v>558645.0087404712</x:v>
+        <x:v>558161.9862245091</x:v>
       </x:c>
       <x:c r="C8" s="108"/>
       <x:c r="D8" s="130" t="str">
-        <x:v>Construction</x:v>
+        <x:v>Consumer</x:v>
       </x:c>
       <x:c r="E8" s="132" t="n">
-        <x:v>56676.95791850734</x:v>
+        <x:v>56386.52830902028</x:v>
       </x:c>
       <x:c r="F8" s="132" t="n">
-        <x:v>41831.82965561585</x:v>
+        <x:v>45194.65609011863</x:v>
       </x:c>
       <x:c r="G8" s="132" t="n">
-        <x:v>76215.77729539698</x:v>
+        <x:v>73791.51077494054</x:v>
       </x:c>
       <x:c r="H8" s="131" t="n">
-        <x:v>751</x:v>
+        <x:v>798</x:v>
       </x:c>
       <x:c r="I8" s="133" t="n">
-        <x:v>0.0806344293</x:v>
+        <x:v>0.0804676388</x:v>
       </x:c>
       <x:c r="J8" s="133" t="n">
-        <x:v>0.1045948194</x:v>
+        <x:v>0.1264962849</x:v>
       </x:c>
       <x:c r="K8" s="134" t="n">
-        <x:v>0.0065019112</x:v>
+        <x:v>0.0064750409</x:v>
       </x:c>
       <x:c r="L8" s="133" t="n">
-        <x:v>0.0156396856</x:v>
+        <x:v>0.0320570166</x:v>
       </x:c>
       <x:c r="M8" s="133" t="n">
-        <x:v>0.8537634137</x:v>
+        <x:v>0.729461539</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -3932,38 +4028,38 @@
         <x:v>Total EAD</x:v>
       </x:c>
       <x:c r="B9" s="132" t="n">
-        <x:v>702887.8163117705</x:v>
+        <x:v>700735.4648341014</x:v>
       </x:c>
       <x:c r="C9" s="108"/>
       <x:c r="D9" s="130" t="str">
         <x:v>Healthcare</x:v>
       </x:c>
       <x:c r="E9" s="132" t="n">
-        <x:v>54065.84992462452</x:v>
+        <x:v>55560.39436053274</x:v>
       </x:c>
       <x:c r="F9" s="132" t="n">
-        <x:v>40331.86011554204</x:v>
+        <x:v>44659.99967842894</x:v>
       </x:c>
       <x:c r="G9" s="132" t="n">
-        <x:v>73907.18002545215</x:v>
+        <x:v>68681.83827448396</x:v>
       </x:c>
       <x:c r="H9" s="131" t="n">
-        <x:v>748</x:v>
+        <x:v>763</x:v>
       </x:c>
       <x:c r="I9" s="133" t="n">
-        <x:v>0.0769196004</x:v>
+        <x:v>0.0792886862</x:v>
       </x:c>
       <x:c r="J9" s="133" t="n">
-        <x:v>0.101426613</x:v>
+        <x:v>0.1177370851</x:v>
       </x:c>
       <x:c r="K9" s="134" t="n">
-        <x:v>0.0059166249</x:v>
+        <x:v>0.0062866958</x:v>
       </x:c>
       <x:c r="L9" s="133" t="n">
-        <x:v>0.0357723532</x:v>
+        <x:v>0.0591812763</x:v>
       </x:c>
       <x:c r="M9" s="133" t="n">
-        <x:v>0.866107059</x:v>
+        <x:v>0.7374324885</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -3971,38 +4067,38 @@
         <x:v>SA Credit RWA</x:v>
       </x:c>
       <x:c r="B10" s="132" t="n">
-        <x:v>406207.69049290236</x:v>
+        <x:v>405323.35943071585</x:v>
       </x:c>
       <x:c r="C10" s="108"/>
       <x:c r="D10" s="130" t="str">
         <x:v>Auto Components</x:v>
       </x:c>
       <x:c r="E10" s="132" t="n">
-        <x:v>52072.79231762107</x:v>
+        <x:v>55206.43975694961</x:v>
       </x:c>
       <x:c r="F10" s="132" t="n">
-        <x:v>37238.740102879274</x:v>
+        <x:v>39097.86430976885</x:v>
       </x:c>
       <x:c r="G10" s="132" t="n">
-        <x:v>67220.0481968937</x:v>
+        <x:v>57473.77884345482</x:v>
       </x:c>
       <x:c r="H10" s="131" t="n">
-        <x:v>770</x:v>
+        <x:v>719</x:v>
       </x:c>
       <x:c r="I10" s="133" t="n">
-        <x:v>0.074084073</x:v>
+        <x:v>0.0787835674</x:v>
       </x:c>
       <x:c r="J10" s="133" t="n">
-        <x:v>0.0922495191</x:v>
+        <x:v>0.0985237926</x:v>
       </x:c>
       <x:c r="K10" s="134" t="n">
-        <x:v>0.0054884499</x:v>
+        <x:v>0.0062068505</x:v>
       </x:c>
       <x:c r="L10" s="133" t="n">
-        <x:v>0.0217333532</x:v>
+        <x:v>0.0189685032</x:v>
       </x:c>
       <x:c r="M10" s="133" t="n">
-        <x:v>0.8584201093</x:v>
+        <x:v>0.7151391872</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -4010,38 +4106,38 @@
         <x:v>IRB Credit RWA</x:v>
       </x:c>
       <x:c r="B11" s="132" t="n">
-        <x:v>728676.4076818405</x:v>
+        <x:v>583349.2328979744</x:v>
       </x:c>
       <x:c r="C11" s="108"/>
       <x:c r="D11" s="130" t="str">
-        <x:v>Consumer</x:v>
+        <x:v>Metals</x:v>
       </x:c>
       <x:c r="E11" s="132" t="n">
-        <x:v>52062.93394994506</x:v>
+        <x:v>53794.76729112122</x:v>
       </x:c>
       <x:c r="F11" s="132" t="n">
-        <x:v>39460.70262409381</x:v>
+        <x:v>41296.49609524937</x:v>
       </x:c>
       <x:c r="G11" s="132" t="n">
-        <x:v>77413.87259869809</x:v>
+        <x:v>56226.87272523917</x:v>
       </x:c>
       <x:c r="H11" s="131" t="n">
-        <x:v>692</x:v>
+        <x:v>748</x:v>
       </x:c>
       <x:c r="I11" s="133" t="n">
-        <x:v>0.0740700475</x:v>
+        <x:v>0.0767690091</x:v>
       </x:c>
       <x:c r="J11" s="133" t="n">
-        <x:v>0.1062390271</x:v>
+        <x:v>0.0963862975</x:v>
       </x:c>
       <x:c r="K11" s="134" t="n">
-        <x:v>0.0054863719</x:v>
+        <x:v>0.0058934808</x:v>
       </x:c>
       <x:c r="L11" s="133" t="n">
-        <x:v>0.0357031892</x:v>
+        <x:v>0.0641568266</x:v>
       </x:c>
       <x:c r="M11" s="133" t="n">
-        <x:v>0.8726246939</x:v>
+        <x:v>0.7062396231</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -4049,38 +4145,38 @@
         <x:v>IRB expected loss</x:v>
       </x:c>
       <x:c r="B12" s="132" t="n">
-        <x:v>13235.315584936732</x:v>
+        <x:v>11753.820884425715</x:v>
       </x:c>
       <x:c r="C12" s="108"/>
       <x:c r="D12" s="130" t="str">
         <x:v>Real Estate</x:v>
       </x:c>
       <x:c r="E12" s="132" t="n">
-        <x:v>51225.30776050267</x:v>
+        <x:v>51375.74011517681</x:v>
       </x:c>
       <x:c r="F12" s="132" t="n">
-        <x:v>39152.741043725706</x:v>
+        <x:v>38375.25759226207</x:v>
       </x:c>
       <x:c r="G12" s="132" t="n">
-        <x:v>72800.36920605261</x:v>
+        <x:v>58473.76140144328</x:v>
       </x:c>
       <x:c r="H12" s="131" t="n">
-        <x:v>692</x:v>
+        <x:v>764</x:v>
       </x:c>
       <x:c r="I12" s="133" t="n">
-        <x:v>0.0728783549</x:v>
+        <x:v>0.073316883</x:v>
       </x:c>
       <x:c r="J12" s="133" t="n">
-        <x:v>0.0999076798</x:v>
+        <x:v>0.1002380017</x:v>
       </x:c>
       <x:c r="K12" s="134" t="n">
-        <x:v>0.0053112546</x:v>
+        <x:v>0.0053753653</x:v>
       </x:c>
       <x:c r="L12" s="133" t="n">
-        <x:v>0.0280689783</x:v>
+        <x:v>0.0187784582</x:v>
       </x:c>
       <x:c r="M12" s="133" t="n">
-        <x:v>0.8594363648</x:v>
+        <x:v>0.6951308116</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -4088,38 +4184,38 @@
         <x:v>Defaulted EAD share</x:v>
       </x:c>
       <x:c r="B13" s="136" t="n">
-        <x:v>0.00911341</x:v>
+        <x:v>0.0116055326</x:v>
       </x:c>
       <x:c r="C13" s="108"/>
       <x:c r="D13" s="130" t="str">
         <x:v>Textiles</x:v>
       </x:c>
       <x:c r="E13" s="132" t="n">
-        <x:v>51096.11604985064</x:v>
+        <x:v>49373.77806757153</x:v>
       </x:c>
       <x:c r="F13" s="132" t="n">
-        <x:v>37158.9299293698</x:v>
+        <x:v>35765.45510411914</x:v>
       </x:c>
       <x:c r="G13" s="132" t="n">
-        <x:v>67516.38567801227</x:v>
+        <x:v>53961.88452084408</x:v>
       </x:c>
       <x:c r="H13" s="131" t="n">
-        <x:v>753</x:v>
+        <x:v>690</x:v>
       </x:c>
       <x:c r="I13" s="133" t="n">
-        <x:v>0.0726945536</x:v>
+        <x:v>0.0704599389</x:v>
       </x:c>
       <x:c r="J13" s="133" t="n">
-        <x:v>0.0926561982</x:v>
+        <x:v>0.0925035664</x:v>
       </x:c>
       <x:c r="K13" s="134" t="n">
-        <x:v>0.0052844981</x:v>
+        <x:v>0.004964603</x:v>
       </x:c>
       <x:c r="L13" s="133" t="n">
-        <x:v>0.0263883161</x:v>
+        <x:v>0.0134214454</x:v>
       </x:c>
       <x:c r="M13" s="133" t="n">
-        <x:v>0.8641609585</x:v>
+        <x:v>0.7068004833</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -4127,34 +4223,34 @@
       <x:c r="B14" s="108"/>
       <x:c r="C14" s="108"/>
       <x:c r="D14" s="130" t="str">
-        <x:v>Metals</x:v>
+        <x:v>IT Services</x:v>
       </x:c>
       <x:c r="E14" s="132" t="n">
-        <x:v>50671.358803696654</x:v>
+        <x:v>48813.3987798572</x:v>
       </x:c>
       <x:c r="F14" s="132" t="n">
-        <x:v>35736.46816151226</x:v>
+        <x:v>36211.72002339181</x:v>
       </x:c>
       <x:c r="G14" s="132" t="n">
-        <x:v>64672.544566003366</x:v>
+        <x:v>48747.04568179307</x:v>
       </x:c>
       <x:c r="H14" s="131" t="n">
-        <x:v>732</x:v>
+        <x:v>713</x:v>
       </x:c>
       <x:c r="I14" s="133" t="n">
-        <x:v>0.0720902506</x:v>
+        <x:v>0.0696602373</x:v>
       </x:c>
       <x:c r="J14" s="133" t="n">
-        <x:v>0.0887534492</x:v>
+        <x:v>0.0835640864</x:v>
       </x:c>
       <x:c r="K14" s="134" t="n">
-        <x:v>0.0051970042</x:v>
+        <x:v>0.0048525487</x:v>
       </x:c>
       <x:c r="L14" s="133" t="n">
-        <x:v>0.0364650645</x:v>
+        <x:v>0.026464078</x:v>
       </x:c>
       <x:c r="M14" s="133" t="n">
-        <x:v>0.8614747978</x:v>
+        <x:v>0.6613784008</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -4162,34 +4258,34 @@
       <x:c r="B15" s="108"/>
       <x:c r="C15" s="108"/>
       <x:c r="D15" s="130" t="str">
-        <x:v>IT Services</x:v>
+        <x:v>Construction</x:v>
       </x:c>
       <x:c r="E15" s="132" t="n">
-        <x:v>46225.33380274554</x:v>
+        <x:v>46076.30833343573</x:v>
       </x:c>
       <x:c r="F15" s="132" t="n">
-        <x:v>35454.61503323175</x:v>
+        <x:v>35244.38448797079</x:v>
       </x:c>
       <x:c r="G15" s="132" t="n">
-        <x:v>65709.94339051725</x:v>
+        <x:v>50542.276874128765</x:v>
       </x:c>
       <x:c r="H15" s="131" t="n">
-        <x:v>710</x:v>
+        <x:v>684</x:v>
       </x:c>
       <x:c r="I15" s="133" t="n">
-        <x:v>0.0657648813</x:v>
+        <x:v>0.065754212</x:v>
       </x:c>
       <x:c r="J15" s="133" t="n">
-        <x:v>0.0901771248</x:v>
+        <x:v>0.0866415417</x:v>
       </x:c>
       <x:c r="K15" s="134" t="n">
-        <x:v>0.0043250196</x:v>
+        <x:v>0.0043236164</x:v>
       </x:c>
       <x:c r="L15" s="133" t="n">
-        <x:v>0.034383143</x:v>
+        <x:v>0.0223150762</x:v>
       </x:c>
       <x:c r="M15" s="133" t="n">
-        <x:v>0.8584900388</x:v>
+        <x:v>0.6770269599</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -4200,31 +4296,31 @@
         <x:v>Households</x:v>
       </x:c>
       <x:c r="E16" s="137" t="n">
-        <x:v>4845.029856473051</x:v>
+        <x:v>4830.272377160793</x:v>
       </x:c>
       <x:c r="F16" s="137" t="n">
-        <x:v>1893.0509857737502</x:v>
+        <x:v>1878.4942582959209</x:v>
       </x:c>
       <x:c r="G16" s="137" t="n">
-        <x:v>1905.1259015397159</x:v>
+        <x:v>1849.1911339571884</x:v>
       </x:c>
       <x:c r="H16" s="138" t="n">
         <x:v>21600</x:v>
       </x:c>
       <x:c r="I16" s="136" t="n">
-        <x:v>0.0068930343</x:v>
+        <x:v>0.0068931467</x:v>
       </x:c>
       <x:c r="J16" s="136" t="n">
-        <x:v>0.002614502</x:v>
+        <x:v>0.0031699555</x:v>
       </x:c>
       <x:c r="K16" s="139" t="n">
-        <x:v>0.0000475139</x:v>
+        <x:v>0.0000475155</x:v>
       </x:c>
       <x:c r="L16" s="136" t="n">
-        <x:v>0.0265328093</x:v>
+        <x:v>0.0253208114</x:v>
       </x:c>
       <x:c r="M16" s="136" t="n">
-        <x:v>0.3646381065</x:v>
+        <x:v>0.3588759676</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -4311,34 +4407,34 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="125" t="str">
-        <x:v>corporate_revolver</x:v>
+        <x:v>Corporate Revolver</x:v>
       </x:c>
       <x:c r="B21" s="127" t="n">
-        <x:v>451656.8611635373</x:v>
+        <x:v>446058.509896505</x:v>
       </x:c>
       <x:c r="C21" s="127" t="n">
-        <x:v>331713.0381324569</x:v>
+        <x:v>332196.40754626686</x:v>
       </x:c>
       <x:c r="D21" s="127" t="n">
-        <x:v>608677.0770615615</x:v>
+        <x:v>491236.5943637679</x:v>
       </x:c>
       <x:c r="E21" s="126" t="n">
         <x:v>3000</x:v>
       </x:c>
       <x:c r="F21" s="128" t="n">
-        <x:v>0.6425731826</x:v>
+        <x:v>0.6365576345</x:v>
       </x:c>
       <x:c r="G21" s="128" t="n">
-        <x:v>0.8353187652</x:v>
+        <x:v>0.8420969235</x:v>
       </x:c>
       <x:c r="H21" s="129" t="n">
-        <x:v>0.412900295</x:v>
+        <x:v>0.405205622</x:v>
       </x:c>
       <x:c r="I21" s="128" t="n">
-        <x:v>0.0270734638</x:v>
+        <x:v>0.0308539897</x:v>
       </x:c>
       <x:c r="J21" s="128" t="n">
-        <x:v>0.8597750019</x:v>
+        <x:v>0.6970631623</x:v>
       </x:c>
       <x:c r="K21" s="108"/>
       <x:c r="L21" s="108"/>
@@ -4346,31 +4442,31 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="130" t="str">
-        <x:v>sovereign_bond</x:v>
+        <x:v>Sovereign Bond</x:v>
       </x:c>
       <x:c r="B22" s="132" t="n">
-        <x:v>136416.9025098093</x:v>
+        <x:v>139386.41947664847</x:v>
       </x:c>
       <x:c r="C22" s="132" t="n">
-        <x:v>21593.660292094177</x:v>
+        <x:v>19020.99985192112</x:v>
       </x:c>
       <x:c r="D22" s="132" t="n">
-        <x:v>28665.82682924301</x:v>
+        <x:v>25475.185787076643</x:v>
       </x:c>
       <x:c r="E22" s="131" t="n">
         <x:v>750</x:v>
       </x:c>
       <x:c r="F22" s="133" t="n">
-        <x:v>0.194080619</x:v>
+        <x:v>0.1989144641</x:v>
       </x:c>
       <x:c r="G22" s="133" t="n">
-        <x:v>0.0393395841</x:v>
+        <x:v>0.0436705568</x:v>
       </x:c>
       <x:c r="H22" s="134" t="n">
-        <x:v>0.0376672867</x:v>
+        <x:v>0.039566964</x:v>
       </x:c>
       <x:c r="I22" s="133" t="n">
-        <x:v>0.0017969369</x:v>
+        <x:v>0.0003817235</x:v>
       </x:c>
       <x:c r="J22" s="133" t="n">
         <x:v>0.7621587156</x:v>
@@ -4381,34 +4477,34 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="130" t="str">
-        <x:v>bank_loan</x:v>
+        <x:v>Bank Loan</x:v>
       </x:c>
       <x:c r="B23" s="132" t="n">
-        <x:v>86527.409619925</x:v>
+        <x:v>86474.13616761977</x:v>
       </x:c>
       <x:c r="C23" s="132" t="n">
-        <x:v>31070.09010510498</x:v>
+        <x:v>29681.62253803385</x:v>
       </x:c>
       <x:c r="D23" s="132" t="n">
-        <x:v>48316.007832624324</x:v>
+        <x:v>24798.62711637545</x:v>
       </x:c>
       <x:c r="E23" s="131" t="n">
         <x:v>1050</x:v>
       </x:c>
       <x:c r="F23" s="133" t="n">
-        <x:v>0.1231027308</x:v>
+        <x:v>0.1234048232</x:v>
       </x:c>
       <x:c r="G23" s="133" t="n">
-        <x:v>0.0663065351</x:v>
+        <x:v>0.0425107735</x:v>
       </x:c>
       <x:c r="H23" s="134" t="n">
-        <x:v>0.0151542823</x:v>
+        <x:v>0.0152287504</x:v>
       </x:c>
       <x:c r="I23" s="133" t="n">
-        <x:v>0.0085432083</x:v>
+        <x:v>0.0100138952</x:v>
       </x:c>
       <x:c r="J23" s="133" t="n">
-        <x:v>0.750331604</x:v>
+        <x:v>0.4091814573</x:v>
       </x:c>
       <x:c r="K23" s="108"/>
       <x:c r="L23" s="108"/>
@@ -4416,34 +4512,34 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="130" t="str">
-        <x:v>sme_revolver</x:v>
+        <x:v>Sme Revolver</x:v>
       </x:c>
       <x:c r="B24" s="132" t="n">
-        <x:v>22244.3296729542</x:v>
+        <x:v>22800.968210256615</x:v>
       </x:c>
       <x:c r="C24" s="132" t="n">
-        <x:v>18760.637671838496</x:v>
+        <x:v>21377.174518654247</x:v>
       </x:c>
       <x:c r="D24" s="132" t="n">
-        <x:v>38268.475394656554</x:v>
+        <x:v>37788.55517175737</x:v>
       </x:c>
       <x:c r="E24" s="131" t="n">
         <x:v>3000</x:v>
       </x:c>
       <x:c r="F24" s="133" t="n">
-        <x:v>0.0316470554</x:v>
+        <x:v>0.0325386246</x:v>
       </x:c>
       <x:c r="G24" s="133" t="n">
-        <x:v>0.0525177912</x:v>
+        <x:v>0.0647786147</x:v>
       </x:c>
       <x:c r="H24" s="134" t="n">
-        <x:v>0.0010015361</x:v>
+        <x:v>0.0010587621</x:v>
       </x:c>
       <x:c r="I24" s="133" t="n">
-        <x:v>0.0459795984</x:v>
+        <x:v>0.0491204748</x:v>
       </x:c>
       <x:c r="J24" s="133" t="n">
-        <x:v>0.9045749948</x:v>
+        <x:v>0.8952487526</x:v>
       </x:c>
       <x:c r="K24" s="108"/>
       <x:c r="L24" s="108"/>
@@ -4451,34 +4547,34 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="130" t="str">
-        <x:v>mortgage</x:v>
+        <x:v>Mortgage</x:v>
       </x:c>
       <x:c r="B25" s="132" t="n">
-        <x:v>4269.50921356602</x:v>
+        <x:v>4269.668168144086</x:v>
       </x:c>
       <x:c r="C25" s="132" t="n">
-        <x:v>1470.0858932068913</x:v>
+        <x:v>1467.2297853842565</x:v>
       </x:c>
       <x:c r="D25" s="132" t="n">
-        <x:v>1282.3197817563369</x:v>
+        <x:v>1267.088586600567</x:v>
       </x:c>
       <x:c r="E25" s="131" t="n">
         <x:v>9600</x:v>
       </x:c>
       <x:c r="F25" s="133" t="n">
-        <x:v>0.0060742399</x:v>
+        <x:v>0.0060931241</x:v>
       </x:c>
       <x:c r="G25" s="133" t="n">
-        <x:v>0.0017597932</x:v>
+        <x:v>0.0021720927</x:v>
       </x:c>
       <x:c r="H25" s="134" t="n">
-        <x:v>0.0000368964</x:v>
+        <x:v>0.0000371262</x:v>
       </x:c>
       <x:c r="I25" s="133" t="n">
-        <x:v>0.0230168471</x:v>
+        <x:v>0.0219817012</x:v>
       </x:c>
       <x:c r="J25" s="133" t="n">
-        <x:v>0.279125169</x:v>
+        <x:v>0.2748254131</x:v>
       </x:c>
       <x:c r="K25" s="108"/>
       <x:c r="L25" s="108"/>
@@ -4486,31 +4582,31 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="130" t="str">
-        <x:v>other</x:v>
+        <x:v>Other</x:v>
       </x:c>
       <x:c r="B26" s="132" t="n">
-        <x:v>1197.2834890715835</x:v>
+        <x:v>1185.1587059108497</x:v>
       </x:c>
       <x:c r="C26" s="132" t="n">
-        <x:v>1177.2133056340365</x:v>
+        <x:v>1168.6607175438987</x:v>
       </x:c>
       <x:c r="D26" s="132" t="n">
-        <x:v>2843.8946622154044</x:v>
+        <x:v>2201.0793250398638</x:v>
       </x:c>
       <x:c r="E26" s="131" t="n">
         <x:v>600</x:v>
       </x:c>
       <x:c r="F26" s="133" t="n">
-        <x:v>0.0017033778</x:v>
+        <x:v>0.0016913069</x:v>
       </x:c>
       <x:c r="G26" s="133" t="n">
-        <x:v>0.0039028225</x:v>
+        <x:v>0.003773176</x:v>
       </x:c>
       <x:c r="H26" s="134" t="n">
-        <x:v>0.0000029015</x:v>
+        <x:v>0.0000028605</x:v>
       </x:c>
       <x:c r="I26" s="133" t="n">
-        <x:v>0.0385917965</x:v>
+        <x:v>0.0336020854</x:v>
       </x:c>
       <x:c r="J26" s="133" t="n">
         <x:v>0.9888634863</x:v>
@@ -4521,31 +4617,31 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="130" t="str">
-        <x:v>personal_loan</x:v>
+        <x:v>Personal Loan</x:v>
       </x:c>
       <x:c r="B27" s="132" t="n">
-        <x:v>497.6717458760974</x:v>
+        <x:v>482.9275557947405</x:v>
       </x:c>
       <x:c r="C27" s="132" t="n">
-        <x:v>369.7520298225129</x:v>
+        <x:v>358.376695887571</x:v>
       </x:c>
       <x:c r="D27" s="132" t="n">
-        <x:v>526.1922652845958</x:v>
+        <x:v>516.0911275685507</x:v>
       </x:c>
       <x:c r="E27" s="131" t="n">
         <x:v>6000</x:v>
       </x:c>
       <x:c r="F27" s="133" t="n">
-        <x:v>0.0007080387</x:v>
+        <x:v>0.0006891724</x:v>
       </x:c>
       <x:c r="G27" s="133" t="n">
-        <x:v>0.0007221206</x:v>
+        <x:v>0.0008847035</x:v>
       </x:c>
       <x:c r="H27" s="134" t="n">
-        <x:v>5.013e-7</x:v>
+        <x:v>4.75e-7</x:v>
       </x:c>
       <x:c r="I27" s="133" t="n">
-        <x:v>0.0518063241</x:v>
+        <x:v>0.049581324</x:v>
       </x:c>
       <x:c r="J27" s="133" t="n">
         <x:v>0.9988634863</x:v>
@@ -4556,31 +4652,31 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="135" t="str">
-        <x:v>credit_card</x:v>
+        <x:v>Credit Card</x:v>
       </x:c>
       <x:c r="B28" s="137" t="n">
-        <x:v>77.84889703093373</x:v>
+        <x:v>77.67665322196703</x:v>
       </x:c>
       <x:c r="C28" s="137" t="n">
-        <x:v>53.21306274434606</x:v>
+        <x:v>52.88777702409341</x:v>
       </x:c>
       <x:c r="D28" s="137" t="n">
-        <x:v>96.61385449878337</x:v>
+        <x:v>66.01141978807071</x:v>
       </x:c>
       <x:c r="E28" s="138" t="n">
         <x:v>6000</x:v>
       </x:c>
       <x:c r="F28" s="136" t="n">
-        <x:v>0.0001107558</x:v>
+        <x:v>0.0001108502</x:v>
       </x:c>
       <x:c r="G28" s="136" t="n">
-        <x:v>0.0001325881</x:v>
+        <x:v>0.0001131593</x:v>
       </x:c>
       <x:c r="H28" s="139" t="n">
         <x:v>1.23e-8</x:v>
       </x:c>
       <x:c r="I28" s="136" t="n">
-        <x:v>0.0577923222</x:v>
+        <x:v>0.0580310597</x:v>
       </x:c>
       <x:c r="J28" s="136" t="n">
         <x:v>1</x:v>
@@ -4688,10 +4784,10 @@
     <x:mergeCell ref="A19:J19"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re5c01dc1da964b37"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0fd5d0e909e4c87"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93972d3ffd3b4945"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c2369b5d7fc4655"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca1d95b8fb894ced"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c2f60a9d31845e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4779,19 +4875,19 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="125" t="str">
-        <x:v>bank</x:v>
+        <x:v>Bank</x:v>
       </x:c>
       <x:c r="B5" s="127" t="n">
-        <x:v>86076.16497439815</x:v>
+        <x:v>85966.04813679571</x:v>
       </x:c>
       <x:c r="C5" s="127" t="n">
-        <x:v>77941.53987925872</x:v>
+        <x:v>78197.27112242617</x:v>
       </x:c>
       <x:c r="D5" s="127" t="n">
-        <x:v>30429.420773156085</x:v>
+        <x:v>29067.4864009404</x:v>
       </x:c>
       <x:c r="E5" s="128" t="n">
-        <x:v>0.3783190067</x:v>
+        <x:v>0.3746397695</x:v>
       </x:c>
       <x:c r="F5" s="108"/>
       <x:c r="G5" s="108"/>
@@ -4803,19 +4899,19 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="130" t="str">
-        <x:v>corporate</x:v>
+        <x:v>Corporate</x:v>
       </x:c>
       <x:c r="B6" s="132" t="n">
-        <x:v>446283.67058253963</x:v>
+        <x:v>435228.34779463586</x:v>
       </x:c>
       <x:c r="C6" s="132" t="n">
-        <x:v>446283.67058253963</x:v>
+        <x:v>435228.34779463586</x:v>
       </x:c>
       <x:c r="D6" s="132" t="n">
-        <x:v>323943.3793049858</x:v>
+        <x:v>318593.53247924795</x:v>
       </x:c>
       <x:c r="E6" s="133" t="n">
-        <x:v>0.7357166948</x:v>
+        <x:v>0.7413683506</x:v>
       </x:c>
       <x:c r="F6" s="108"/>
       <x:c r="G6" s="108"/>
@@ -4827,19 +4923,19 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="130" t="str">
-        <x:v>corporate_sme</x:v>
+        <x:v>Corporate Sme</x:v>
       </x:c>
       <x:c r="B7" s="132" t="n">
-        <x:v>21855.870140243373</x:v>
+        <x:v>26066.645920357958</x:v>
       </x:c>
       <x:c r="C7" s="132" t="n">
-        <x:v>21855.870140243373</x:v>
+        <x:v>26066.645920357958</x:v>
       </x:c>
       <x:c r="D7" s="132" t="n">
-        <x:v>18194.208263272943</x:v>
+        <x:v>23713.936071489585</x:v>
       </x:c>
       <x:c r="E7" s="133" t="n">
-        <x:v>0.85</x:v>
+        <x:v>0.951691989</x:v>
       </x:c>
       <x:c r="F7" s="108"/>
       <x:c r="G7" s="108"/>
@@ -4851,16 +4947,16 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="130" t="str">
-        <x:v>defaulted</x:v>
+        <x:v>Defaulted</x:v>
       </x:c>
       <x:c r="B8" s="132" t="n">
-        <x:v>6405.704843286997</x:v>
+        <x:v>8132.40826055647</x:v>
       </x:c>
       <x:c r="C8" s="132" t="n">
-        <x:v>6405.704843286997</x:v>
+        <x:v>8057.300333152173</x:v>
       </x:c>
       <x:c r="D8" s="132" t="n">
-        <x:v>9265.201245969505</x:v>
+        <x:v>11969.24894388547</x:v>
       </x:c>
       <x:c r="E8" s="133" t="n">
         <x:v>1.5</x:v>
@@ -4875,16 +4971,16 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="130" t="str">
-        <x:v>other</x:v>
+        <x:v>Other</x:v>
       </x:c>
       <x:c r="B9" s="132" t="n">
-        <x:v>1186.5880051395955</x:v>
+        <x:v>1168.2712109863826</x:v>
       </x:c>
       <x:c r="C9" s="132" t="n">
-        <x:v>1186.5880051395955</x:v>
+        <x:v>1168.2712109863826</x:v>
       </x:c>
       <x:c r="D9" s="132" t="n">
-        <x:v>1161.1700797360543</x:v>
+        <x:v>1143.3294751571984</x:v>
       </x:c>
       <x:c r="E9" s="133" t="n">
         <x:v>1</x:v>
@@ -4899,16 +4995,16 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="130" t="str">
-        <x:v>regulatory_retail</x:v>
+        <x:v>Regulatory Retail</x:v>
       </x:c>
       <x:c r="B10" s="132" t="n">
-        <x:v>488.5652336979505</x:v>
+        <x:v>475.23306052162934</x:v>
       </x:c>
       <x:c r="C10" s="132" t="n">
-        <x:v>488.5652336979505</x:v>
+        <x:v>475.23306052162934</x:v>
       </x:c>
       <x:c r="D10" s="132" t="n">
-        <x:v>356.4014251673766</x:v>
+        <x:v>347.0928942833718</x:v>
       </x:c>
       <x:c r="E10" s="133" t="n">
         <x:v>0.75</x:v>
@@ -4923,19 +5019,19 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="130" t="str">
-        <x:v>residential_real_estate</x:v>
+        <x:v>Residential Real Estate</x:v>
       </x:c>
       <x:c r="B11" s="132" t="n">
-        <x:v>4231.114864326715</x:v>
+        <x:v>4235.829879346015</x:v>
       </x:c>
       <x:c r="C11" s="132" t="n">
-        <x:v>4231.114864326715</x:v>
+        <x:v>4235.829879346015</x:v>
       </x:c>
       <x:c r="D11" s="132" t="n">
-        <x:v>1412.8559740037292</x:v>
+        <x:v>1416.9298770252751</x:v>
       </x:c>
       <x:c r="E11" s="133" t="n">
-        <x:v>0.3387896617</x:v>
+        <x:v>0.3387464537</x:v>
       </x:c>
       <x:c r="F11" s="108"/>
       <x:c r="G11" s="108"/>
@@ -4947,16 +5043,16 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="130" t="str">
-        <x:v>retail_transactor</x:v>
+        <x:v>Retail Transactor</x:v>
       </x:c>
       <x:c r="B12" s="132" t="n">
-        <x:v>16.595837881879238</x:v>
+        <x:v>16.929704837020306</x:v>
       </x:c>
       <x:c r="C12" s="132" t="n">
-        <x:v>16.595837881879238</x:v>
+        <x:v>16.929704837020306</x:v>
       </x:c>
       <x:c r="D12" s="132" t="n">
-        <x:v>7.336783659514953</x:v>
+        <x:v>7.456961655098778</x:v>
       </x:c>
       <x:c r="E12" s="133" t="n">
         <x:v>0.45</x:v>
@@ -4971,16 +5067,16 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="130" t="str">
-        <x:v>revolving_retail</x:v>
+        <x:v>Revolving Retail</x:v>
       </x:c>
       <x:c r="B13" s="132" t="n">
-        <x:v>59.876394793925485</x:v>
+        <x:v>59.331389416021715</x:v>
       </x:c>
       <x:c r="C13" s="132" t="n">
-        <x:v>59.876394793925485</x:v>
+        <x:v>59.331389416021715</x:v>
       </x:c>
       <x:c r="D13" s="132" t="n">
-        <x:v>43.91196237781136</x:v>
+        <x:v>43.34647511042866</x:v>
       </x:c>
       <x:c r="E13" s="133" t="n">
         <x:v>0.75</x:v>
@@ -4995,19 +5091,19 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="135" t="str">
-        <x:v>sovereign</x:v>
+        <x:v>Sovereign</x:v>
       </x:c>
       <x:c r="B14" s="137" t="n">
-        <x:v>136283.66543546217</x:v>
+        <x:v>139386.41947664847</x:v>
       </x:c>
       <x:c r="C14" s="137" t="n">
-        <x:v>136283.66543546217</x:v>
+        <x:v>139386.41947664847</x:v>
       </x:c>
       <x:c r="D14" s="137" t="n">
-        <x:v>21393.80468057351</x:v>
+        <x:v>19020.99985192112</x:v>
       </x:c>
       <x:c r="E14" s="136" t="n">
-        <x:v>0.1581550802</x:v>
+        <x:v>0.1392</x:v>
       </x:c>
       <x:c r="F14" s="108"/>
       <x:c r="G14" s="108"/>
@@ -5025,7 +5121,7 @@
       <x:c r="C15" s="145"/>
       <x:c r="D15" s="145" t="n">
         <x:f>SUM(D5:D14)</x:f>
-        <x:v>406207.6904929024</x:v>
+        <x:v>405323.3594307159</x:v>
       </x:c>
       <x:c r="E15" s="144"/>
       <x:c r="F15" s="108"/>
@@ -5044,7 +5140,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb98be1ff5dd64fd4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re71978512a644b92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5135,22 +5231,22 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="125" t="str">
-        <x:v>bank</x:v>
+        <x:v>Bank</x:v>
       </x:c>
       <x:c r="B5" s="127" t="n">
-        <x:v>86076.16497439815</x:v>
+        <x:v>85966.04813679571</x:v>
       </x:c>
       <x:c r="C5" s="128" t="n">
-        <x:v>0.0028724928</x:v>
+        <x:v>0.0041627469</x:v>
       </x:c>
       <x:c r="D5" s="128" t="n">
-        <x:v>0.7481433813</x:v>
+        <x:v>0.4093333679</x:v>
       </x:c>
       <x:c r="E5" s="127" t="n">
-        <x:v>217.51884219352294</x:v>
+        <x:v>133.74000465018094</x:v>
       </x:c>
       <x:c r="F5" s="127" t="n">
-        <x:v>48316.007832624324</x:v>
+        <x:v>24798.62711637545</x:v>
       </x:c>
       <x:c r="G5" s="108"/>
       <x:c r="H5" s="108"/>
@@ -5161,22 +5257,22 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="130" t="str">
-        <x:v>corporate</x:v>
+        <x:v>Corporate</x:v>
       </x:c>
       <x:c r="B6" s="132" t="n">
-        <x:v>474975.03644523985</x:v>
+        <x:v>462700.5320184297</x:v>
       </x:c>
       <x:c r="C6" s="133" t="n">
-        <x:v>0.0151038111</x:v>
+        <x:v>0.0149835222</x:v>
       </x:c>
       <x:c r="D6" s="133" t="n">
-        <x:v>0.8565702577</x:v>
+        <x:v>0.7057635631</x:v>
       </x:c>
       <x:c r="E6" s="132" t="n">
-        <x:v>6373.495212371627</x:v>
+        <x:v>4926.029160623198</x:v>
       </x:c>
       <x:c r="F6" s="132" t="n">
-        <x:v>608677.0770615615</x:v>
+        <x:v>484224.5892909211</x:v>
       </x:c>
       <x:c r="G6" s="108"/>
       <x:c r="H6" s="108"/>
@@ -5187,22 +5283,22 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="130" t="str">
-        <x:v>corporate_sme</x:v>
+        <x:v>Corporate Sme</x:v>
       </x:c>
       <x:c r="B7" s="132" t="n">
-        <x:v>23902.488465914797</x:v>
+        <x:v>28549.71908532937</x:v>
       </x:c>
       <x:c r="C7" s="133" t="n">
-        <x:v>0.0289094186</x:v>
+        <x:v>0.030840804</x:v>
       </x:c>
       <x:c r="D7" s="133" t="n">
-        <x:v>0.9017523702</x:v>
+        <x:v>0.8959864016</x:v>
       </x:c>
       <x:c r="E7" s="132" t="n">
-        <x:v>627.4723073643232</x:v>
+        <x:v>788.7907145313042</x:v>
       </x:c>
       <x:c r="F7" s="132" t="n">
-        <x:v>38268.475394656554</x:v>
+        <x:v>44800.56024460412</x:v>
       </x:c>
       <x:c r="G7" s="108"/>
       <x:c r="H7" s="108"/>
@@ -5213,19 +5309,19 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="130" t="str">
-        <x:v>defaulted</x:v>
+        <x:v>Defaulted</x:v>
       </x:c>
       <x:c r="B8" s="132" t="n">
-        <x:v>6846.527818410888</x:v>
+        <x:v>8626.483206591412</x:v>
       </x:c>
       <x:c r="C8" s="133" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="133" t="n">
-        <x:v>0.8286464016</x:v>
+        <x:v>0.6728266024</x:v>
       </x:c>
       <x:c r="E8" s="132" t="n">
-        <x:v>5856.790243326718</x:v>
+        <x:v>5804.127386304351</x:v>
       </x:c>
       <x:c r="F8" s="132" t="n">
         <x:v>0</x:v>
@@ -5239,22 +5335,22 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="130" t="str">
-        <x:v>other</x:v>
+        <x:v>Other</x:v>
       </x:c>
       <x:c r="B9" s="132" t="n">
-        <x:v>1296.7126752615732</x:v>
+        <x:v>1275.2483142732424</x:v>
       </x:c>
       <x:c r="C9" s="133" t="n">
-        <x:v>0.0316541315</x:v>
+        <x:v>0.0195483437</x:v>
       </x:c>
       <x:c r="D9" s="133" t="n">
         <x:v>0.9888634863</x:v>
       </x:c>
       <x:c r="E9" s="132" t="n">
-        <x:v>38.16953584072139</x:v>
+        <x:v>24.651370267018297</x:v>
       </x:c>
       <x:c r="F9" s="132" t="n">
-        <x:v>2843.8946622154044</x:v>
+        <x:v>2201.0793250398638</x:v>
       </x:c>
       <x:c r="G9" s="108"/>
       <x:c r="H9" s="108"/>
@@ -5265,22 +5361,22 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="130" t="str">
-        <x:v>regulatory_retail</x:v>
+        <x:v>Regulatory Retail</x:v>
       </x:c>
       <x:c r="B10" s="132" t="n">
-        <x:v>488.5652336979505</x:v>
+        <x:v>475.23306052162934</x:v>
       </x:c>
       <x:c r="C10" s="133" t="n">
-        <x:v>0.0341651598</x:v>
+        <x:v>0.0341931016</x:v>
       </x:c>
       <x:c r="D10" s="133" t="n">
         <x:v>0.9988634863</x:v>
       </x:c>
       <x:c r="E10" s="132" t="n">
-        <x:v>16.657079068576024</x:v>
+        <x:v>16.231224335542773</x:v>
       </x:c>
       <x:c r="F10" s="132" t="n">
-        <x:v>526.1922652845958</x:v>
+        <x:v>516.0911275685507</x:v>
       </x:c>
       <x:c r="G10" s="108"/>
       <x:c r="H10" s="108"/>
@@ -5291,22 +5387,22 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="130" t="str">
-        <x:v>residential_real_estate</x:v>
+        <x:v>Residential Real Estate</x:v>
       </x:c>
       <x:c r="B11" s="132" t="n">
-        <x:v>4231.114864326715</x:v>
+        <x:v>4235.829879346015</x:v>
       </x:c>
       <x:c r="C11" s="133" t="n">
-        <x:v>0.0140550011</x:v>
+        <x:v>0.0141687185</x:v>
       </x:c>
       <x:c r="D11" s="133" t="n">
-        <x:v>0.278715329</x:v>
+        <x:v>0.2749120394</x:v>
       </x:c>
       <x:c r="E11" s="132" t="n">
-        <x:v>16.63265552015742</x:v>
+        <x:v>16.42794170851161</x:v>
       </x:c>
       <x:c r="F11" s="132" t="n">
-        <x:v>1282.3197817563369</x:v>
+        <x:v>1267.088586600567</x:v>
       </x:c>
       <x:c r="G11" s="108"/>
       <x:c r="H11" s="108"/>
@@ -5317,22 +5413,22 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="130" t="str">
-        <x:v>retail_transactor</x:v>
+        <x:v>Retail Transactor</x:v>
       </x:c>
       <x:c r="B12" s="132" t="n">
-        <x:v>17.551111631538326</x:v>
+        <x:v>17.915730026479636</x:v>
       </x:c>
       <x:c r="C12" s="133" t="n">
-        <x:v>0.04055152</x:v>
+        <x:v>0.0397647667</x:v>
       </x:c>
       <x:c r="D12" s="133" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E12" s="132" t="n">
-        <x:v>0.6898758379900805</x:v>
+        <x:v>0.7124148249269857</x:v>
       </x:c>
       <x:c r="F12" s="132" t="n">
-        <x:v>45.00971625825575</x:v>
+        <x:v>14.430221176662805</x:v>
       </x:c>
       <x:c r="G12" s="108"/>
       <x:c r="H12" s="108"/>
@@ -5343,22 +5439,22 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="130" t="str">
-        <x:v>revolving_retail</x:v>
+        <x:v>Revolving Retail</x:v>
       </x:c>
       <x:c r="B13" s="132" t="n">
-        <x:v>63.291730164368914</x:v>
+        <x:v>62.70139786595153</x:v>
       </x:c>
       <x:c r="C13" s="133" t="n">
-        <x:v>0.040444861</x:v>
+        <x:v>0.0408034732</x:v>
       </x:c>
       <x:c r="D13" s="133" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E13" s="132" t="n">
-        <x:v>2.607708694235685</x:v>
+        <x:v>2.5584348064131426</x:v>
       </x:c>
       <x:c r="F13" s="132" t="n">
-        <x:v>51.60413824052762</x:v>
+        <x:v>51.581198611407906</x:v>
       </x:c>
       <x:c r="G13" s="108"/>
       <x:c r="H13" s="108"/>
@@ -5369,22 +5465,22 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="135" t="str">
-        <x:v>sovereign</x:v>
+        <x:v>Sovereign</x:v>
       </x:c>
       <x:c r="B14" s="137" t="n">
-        <x:v>136283.66543546217</x:v>
+        <x:v>139386.41947664847</x:v>
       </x:c>
       <x:c r="C14" s="136" t="n">
-        <x:v>0.000849746</x:v>
+        <x:v>0.0003817235</x:v>
       </x:c>
       <x:c r="D14" s="136" t="n">
         <x:v>0.7621587156</x:v>
       </x:c>
       <x:c r="E14" s="137" t="n">
-        <x:v>85.28212471886066</x:v>
+        <x:v>40.552232374268954</x:v>
       </x:c>
       <x:c r="F14" s="137" t="n">
-        <x:v>28665.82682924301</x:v>
+        <x:v>25475.185787076643</x:v>
       </x:c>
       <x:c r="G14" s="108"/>
       <x:c r="H14" s="108"/>
@@ -5403,7 +5499,7 @@
       <x:c r="E15" s="145"/>
       <x:c r="F15" s="145" t="n">
         <x:f>SUM(F5:F14)</x:f>
-        <x:v>728676.4076818406</x:v>
+        <x:v>583349.2328979743</x:v>
       </x:c>
       <x:c r="G15" s="108"/>
       <x:c r="H15" s="108"/>
@@ -5420,7 +5516,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb06bf05ae3454f73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69c5d6a6e5b2477a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5434,6 +5530,9 @@
     <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -5508,19 +5607,21 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="125" t="str">
-        <x:v>bank</x:v>
+        <x:v>Bank</x:v>
       </x:c>
       <x:c r="B5" s="127" t="n">
-        <x:v>30429.420773156085</x:v>
+        <x:v>29067.4864009404</x:v>
       </x:c>
       <x:c r="C5" s="127" t="n">
-        <x:v>48316.007832624324</x:v>
+        <x:v>24798.62711637545</x:v>
       </x:c>
       <x:c r="D5" s="127" t="n">
-        <x:v>17886.58705946824</x:v>
+        <x:f>C5-B5</x:f>
+        <x:v>-4268.859284564951</x:v>
       </x:c>
       <x:c r="E5" s="146" t="n">
-        <x:v>1.5878057026720418</x:v>
+        <x:f>IF(B5=0,0,C5/B5)</x:f>
+        <x:v>0.8531397168065126</x:v>
       </x:c>
       <x:c r="F5" s="108"/>
       <x:c r="G5" s="108"/>
@@ -5532,19 +5633,21 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="130" t="str">
-        <x:v>corporate</x:v>
+        <x:v>Corporate</x:v>
       </x:c>
       <x:c r="B6" s="132" t="n">
-        <x:v>323943.3793049858</x:v>
+        <x:v>318593.53247924795</x:v>
       </x:c>
       <x:c r="C6" s="132" t="n">
-        <x:v>608677.0770615615</x:v>
+        <x:v>484224.5892909211</x:v>
       </x:c>
       <x:c r="D6" s="132" t="n">
-        <x:v>284733.6977565757</x:v>
+        <x:f>C6-B6</x:f>
+        <x:v>165631.05681167316</x:v>
       </x:c>
       <x:c r="E6" s="147" t="n">
-        <x:v>1.8789613122128512</x:v>
+        <x:f>IF(B6=0,0,C6/B6)</x:f>
+        <x:v>1.5198820438153802</x:v>
       </x:c>
       <x:c r="F6" s="108"/>
       <x:c r="G6" s="108"/>
@@ -5556,19 +5659,21 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="130" t="str">
-        <x:v>corporate_sme</x:v>
+        <x:v>Corporate Sme</x:v>
       </x:c>
       <x:c r="B7" s="132" t="n">
-        <x:v>18194.208263272943</x:v>
+        <x:v>23713.936071489585</x:v>
       </x:c>
       <x:c r="C7" s="132" t="n">
-        <x:v>38268.475394656554</x:v>
+        <x:v>44800.56024460412</x:v>
       </x:c>
       <x:c r="D7" s="132" t="n">
-        <x:v>20074.26713138361</x:v>
+        <x:f>C7-B7</x:f>
+        <x:v>21086.62417311454</x:v>
       </x:c>
       <x:c r="E7" s="147" t="n">
-        <x:v>2.1033328211321938</x:v>
+        <x:f>IF(B7=0,0,C7/B7)</x:f>
+        <x:v>1.889208105712414</x:v>
       </x:c>
       <x:c r="F7" s="108"/>
       <x:c r="G7" s="108"/>
@@ -5580,18 +5685,20 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="130" t="str">
-        <x:v>defaulted</x:v>
+        <x:v>Defaulted</x:v>
       </x:c>
       <x:c r="B8" s="132" t="n">
-        <x:v>9265.201245969505</x:v>
+        <x:v>11969.24894388547</x:v>
       </x:c>
       <x:c r="C8" s="132" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="132" t="n">
-        <x:v>-9265.201245969505</x:v>
+        <x:f>C8-B8</x:f>
+        <x:v>-11969.24894388547</x:v>
       </x:c>
       <x:c r="E8" s="147" t="n">
+        <x:f>IF(B8=0,0,C8/B8)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F8" s="108"/>
@@ -5604,19 +5711,21 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="130" t="str">
-        <x:v>other</x:v>
+        <x:v>Other</x:v>
       </x:c>
       <x:c r="B9" s="132" t="n">
-        <x:v>1161.1700797360543</x:v>
+        <x:v>1143.3294751571984</x:v>
       </x:c>
       <x:c r="C9" s="132" t="n">
-        <x:v>2843.8946622154044</x:v>
+        <x:v>2201.0793250398638</x:v>
       </x:c>
       <x:c r="D9" s="132" t="n">
-        <x:v>1682.7245824793501</x:v>
+        <x:f>C9-B9</x:f>
+        <x:v>1057.7498498826653</x:v>
       </x:c>
       <x:c r="E9" s="147" t="n">
-        <x:v>2.4491628847876017</x:v>
+        <x:f>IF(B9=0,0,C9/B9)</x:f>
+        <x:v>1.9251487632095143</x:v>
       </x:c>
       <x:c r="F9" s="108"/>
       <x:c r="G9" s="108"/>
@@ -5628,19 +5737,21 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="130" t="str">
-        <x:v>regulatory_retail</x:v>
+        <x:v>Regulatory Retail</x:v>
       </x:c>
       <x:c r="B10" s="132" t="n">
-        <x:v>356.4014251673766</x:v>
+        <x:v>347.0928942833718</x:v>
       </x:c>
       <x:c r="C10" s="132" t="n">
-        <x:v>526.1922652845958</x:v>
+        <x:v>516.0911275685507</x:v>
       </x:c>
       <x:c r="D10" s="132" t="n">
-        <x:v>169.7908401172192</x:v>
+        <x:f>C10-B10</x:f>
+        <x:v>168.99823328517897</x:v>
       </x:c>
       <x:c r="E10" s="147" t="n">
-        <x:v>1.4764033702656505</x:v>
+        <x:f>IF(B10=0,0,C10/B10)</x:f>
+        <x:v>1.4868962634170388</x:v>
       </x:c>
       <x:c r="F10" s="108"/>
       <x:c r="G10" s="108"/>
@@ -5652,19 +5763,21 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="130" t="str">
-        <x:v>residential_real_estate</x:v>
+        <x:v>Residential Real Estate</x:v>
       </x:c>
       <x:c r="B11" s="132" t="n">
-        <x:v>1412.8559740037292</x:v>
+        <x:v>1416.9298770252751</x:v>
       </x:c>
       <x:c r="C11" s="132" t="n">
-        <x:v>1282.3197817563369</x:v>
+        <x:v>1267.088586600567</x:v>
       </x:c>
       <x:c r="D11" s="132" t="n">
-        <x:v>-130.53619224739236</x:v>
+        <x:f>C11-B11</x:f>
+        <x:v>-149.84129042470818</x:v>
       </x:c>
       <x:c r="E11" s="147" t="n">
-        <x:v>0.9076082809223074</x:v>
+        <x:f>IF(B11=0,0,C11/B11)</x:f>
+        <x:v>0.8942493253517335</x:v>
       </x:c>
       <x:c r="F11" s="108"/>
       <x:c r="G11" s="108"/>
@@ -5676,19 +5789,21 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="130" t="str">
-        <x:v>retail_transactor</x:v>
+        <x:v>Retail Transactor</x:v>
       </x:c>
       <x:c r="B12" s="132" t="n">
-        <x:v>7.336783659514953</x:v>
+        <x:v>7.456961655098778</x:v>
       </x:c>
       <x:c r="C12" s="132" t="n">
-        <x:v>45.00971625825575</x:v>
+        <x:v>14.430221176662805</x:v>
       </x:c>
       <x:c r="D12" s="132" t="n">
-        <x:v>37.6729325987408</x:v>
+        <x:f>C12-B12</x:f>
+        <x:v>6.973259521564027</x:v>
       </x:c>
       <x:c r="E12" s="147" t="n">
-        <x:v>6.134802162236771</x:v>
+        <x:f>IF(B12=0,0,C12/B12)</x:f>
+        <x:v>1.9351341530361748</x:v>
       </x:c>
       <x:c r="F12" s="108"/>
       <x:c r="G12" s="108"/>
@@ -5700,19 +5815,21 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="130" t="str">
-        <x:v>revolving_retail</x:v>
+        <x:v>Revolving Retail</x:v>
       </x:c>
       <x:c r="B13" s="132" t="n">
-        <x:v>43.91196237781136</x:v>
+        <x:v>43.34647511042866</x:v>
       </x:c>
       <x:c r="C13" s="132" t="n">
-        <x:v>51.60413824052762</x:v>
+        <x:v>51.581198611407906</x:v>
       </x:c>
       <x:c r="D13" s="132" t="n">
-        <x:v>7.692175862716255</x:v>
+        <x:f>C13-B13</x:f>
+        <x:v>8.234723500979243</x:v>
       </x:c>
       <x:c r="E13" s="147" t="n">
-        <x:v>1.1751726738271004</x:v>
+        <x:f>IF(B13=0,0,C13/B13)</x:f>
+        <x:v>1.1899744668972647</x:v>
       </x:c>
       <x:c r="F13" s="108"/>
       <x:c r="G13" s="108"/>
@@ -5724,19 +5841,21 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="135" t="str">
-        <x:v>sovereign</x:v>
+        <x:v>Sovereign</x:v>
       </x:c>
       <x:c r="B14" s="137" t="n">
-        <x:v>21393.80468057351</x:v>
+        <x:v>19020.99985192112</x:v>
       </x:c>
       <x:c r="C14" s="137" t="n">
-        <x:v>28665.82682924301</x:v>
+        <x:v>25475.185787076643</x:v>
       </x:c>
       <x:c r="D14" s="137" t="n">
-        <x:v>7272.022148669501</x:v>
+        <x:f>C14-B14</x:f>
+        <x:v>6454.185935155525</x:v>
       </x:c>
       <x:c r="E14" s="148" t="n">
-        <x:v>1.3399125240809928</x:v>
+        <x:f>IF(B14=0,0,C14/B14)</x:f>
+        <x:v>1.3393189624836495</x:v>
       </x:c>
       <x:c r="F14" s="108"/>
       <x:c r="G14" s="108"/>
@@ -5800,13 +5919,13 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="125" t="str">
-        <x:v>base</x:v>
+        <x:v>Base</x:v>
       </x:c>
       <x:c r="B18" s="125" t="str">
         <x:v>SA Credit RWA</x:v>
       </x:c>
       <x:c r="C18" s="127" t="n">
-        <x:v>406207.69049290236</x:v>
+        <x:v>405323.35943071585</x:v>
       </x:c>
       <x:c r="D18" s="149" t="b">
         <x:v>0</x:v>
@@ -5822,13 +5941,13 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="130" t="str">
-        <x:v>base</x:v>
+        <x:v>Base</x:v>
       </x:c>
       <x:c r="B19" s="130" t="str">
         <x:v>IRB Credit RWA</x:v>
       </x:c>
       <x:c r="C19" s="132" t="n">
-        <x:v>728676.4076818405</x:v>
+        <x:v>583349.2328979744</x:v>
       </x:c>
       <x:c r="D19" s="150" t="b">
         <x:v>0</x:v>
@@ -5844,13 +5963,13 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="130" t="str">
-        <x:v>base</x:v>
+        <x:v>Base</x:v>
       </x:c>
       <x:c r="B20" s="130" t="str">
-        <x:v>Standardised aggregate RWA base</x:v>
+        <x:v>Standardised Aggregate RWA Base</x:v>
       </x:c>
       <x:c r="C20" s="132" t="n">
-        <x:v>431207.69049290236</x:v>
+        <x:v>430323.35943071585</x:v>
       </x:c>
       <x:c r="D20" s="150" t="b">
         <x:v>0</x:v>
@@ -5858,21 +5977,27 @@
       <x:c r="E20" s="108"/>
       <x:c r="F20" s="108"/>
       <x:c r="G20" s="108"/>
-      <x:c r="H20" s="108"/>
-      <x:c r="I20" s="108"/>
-      <x:c r="J20" s="108"/>
+      <x:c r="H20" s="175" t="str">
+        <x:v>Exposure Class</x:v>
+      </x:c>
+      <x:c r="I20" s="175" t="str">
+        <x:v>SA RWA / EAD</x:v>
+      </x:c>
+      <x:c r="J20" s="175" t="str">
+        <x:v>IRB RWA / EAD</x:v>
+      </x:c>
       <x:c r="K20" s="108"/>
       <x:c r="L20" s="108"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="130" t="str">
-        <x:v>base</x:v>
+        <x:v>Base</x:v>
       </x:c>
       <x:c r="B21" s="130" t="str">
-        <x:v>Pre-floor model aggregate RWA</x:v>
+        <x:v>Pre-Floor Model Aggregate RWA</x:v>
       </x:c>
       <x:c r="C21" s="132" t="n">
-        <x:v>753676.4076818405</x:v>
+        <x:v>608349.2328979744</x:v>
       </x:c>
       <x:c r="D21" s="150" t="b">
         <x:v>0</x:v>
@@ -5880,18 +6005,24 @@
       <x:c r="E21" s="108"/>
       <x:c r="F21" s="108"/>
       <x:c r="G21" s="108"/>
-      <x:c r="H21" s="108"/>
-      <x:c r="I21" s="108"/>
-      <x:c r="J21" s="108"/>
+      <x:c r="H21" s="108" t="str">
+        <x:v>Bank</x:v>
+      </x:c>
+      <x:c r="I21" s="173" t="n">
+        <x:v>0.371719958813296</x:v>
+      </x:c>
+      <x:c r="J21" s="173" t="n">
+        <x:v>0.28847001407944206</x:v>
+      </x:c>
       <x:c r="K21" s="108"/>
       <x:c r="L21" s="108"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="130" t="str">
-        <x:v>base</x:v>
+        <x:v>Base</x:v>
       </x:c>
       <x:c r="B22" s="130" t="str">
-        <x:v>Output-floor rate</x:v>
+        <x:v>Output-Floor Rate</x:v>
       </x:c>
       <x:c r="C22" s="133" t="n">
         <x:v>0.65</x:v>
@@ -5902,21 +6033,27 @@
       <x:c r="E22" s="108"/>
       <x:c r="F22" s="108"/>
       <x:c r="G22" s="108"/>
-      <x:c r="H22" s="108"/>
-      <x:c r="I22" s="108"/>
-      <x:c r="J22" s="108"/>
+      <x:c r="H22" s="108" t="str">
+        <x:v>Corporate</x:v>
+      </x:c>
+      <x:c r="I22" s="173" t="n">
+        <x:v>0.7320146633223843</x:v>
+      </x:c>
+      <x:c r="J22" s="173" t="n">
+        <x:v>1.0465183326645366</x:v>
+      </x:c>
       <x:c r="K22" s="108"/>
       <x:c r="L22" s="108"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="130" t="str">
-        <x:v>base</x:v>
+        <x:v>Base</x:v>
       </x:c>
       <x:c r="B23" s="130" t="str">
-        <x:v>Output-floor amount</x:v>
+        <x:v>Output-Floor Amount</x:v>
       </x:c>
       <x:c r="C23" s="132" t="n">
-        <x:v>280284.99882038654</x:v>
+        <x:v>279710.18362996535</x:v>
       </x:c>
       <x:c r="D23" s="150" t="b">
         <x:v>0</x:v>
@@ -5924,21 +6061,27 @@
       <x:c r="E23" s="108"/>
       <x:c r="F23" s="108"/>
       <x:c r="G23" s="108"/>
-      <x:c r="H23" s="108"/>
-      <x:c r="I23" s="108"/>
-      <x:c r="J23" s="108"/>
+      <x:c r="H23" s="108" t="str">
+        <x:v>Corporate SME</x:v>
+      </x:c>
+      <x:c r="I23" s="173" t="n">
+        <x:v>0.9097425170826863</x:v>
+      </x:c>
+      <x:c r="J23" s="173" t="n">
+        <x:v>1.5692119460336633</x:v>
+      </x:c>
       <x:c r="K23" s="108"/>
       <x:c r="L23" s="108"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="130" t="str">
-        <x:v>base</x:v>
+        <x:v>Base</x:v>
       </x:c>
       <x:c r="B24" s="130" t="str">
-        <x:v>Final aggregate RWA</x:v>
+        <x:v>Final Aggregate RWA</x:v>
       </x:c>
       <x:c r="C24" s="132" t="n">
-        <x:v>753676.4076818405</x:v>
+        <x:v>608349.2328979744</x:v>
       </x:c>
       <x:c r="D24" s="150" t="b">
         <x:v>0</x:v>
@@ -5946,18 +6089,24 @@
       <x:c r="E24" s="108"/>
       <x:c r="F24" s="108"/>
       <x:c r="G24" s="108"/>
-      <x:c r="H24" s="108"/>
-      <x:c r="I24" s="108"/>
-      <x:c r="J24" s="108"/>
+      <x:c r="H24" s="108" t="str">
+        <x:v>Defaulted</x:v>
+      </x:c>
+      <x:c r="I24" s="173" t="n">
+        <x:v>1.485516047433082</x:v>
+      </x:c>
+      <x:c r="J24" s="173" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="K24" s="108"/>
       <x:c r="L24" s="108"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="130" t="str">
-        <x:v>base</x:v>
+        <x:v>Base</x:v>
       </x:c>
       <x:c r="B25" s="130" t="str">
-        <x:v>Floor uplift</x:v>
+        <x:v>Floor Uplift</x:v>
       </x:c>
       <x:c r="C25" s="132" t="n">
         <x:v>0</x:v>
@@ -5968,21 +6117,27 @@
       <x:c r="E25" s="108"/>
       <x:c r="F25" s="108"/>
       <x:c r="G25" s="108"/>
-      <x:c r="H25" s="108"/>
-      <x:c r="I25" s="108"/>
-      <x:c r="J25" s="108"/>
+      <x:c r="H25" s="108" t="str">
+        <x:v>Other</x:v>
+      </x:c>
+      <x:c r="I25" s="173" t="n">
+        <x:v>0.9786507314443488</x:v>
+      </x:c>
+      <x:c r="J25" s="173" t="n">
+        <x:v>1.7260005760480048</x:v>
+      </x:c>
       <x:c r="K25" s="108"/>
       <x:c r="L25" s="108"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="130" t="str">
-        <x:v>adverse</x:v>
+        <x:v>Adverse</x:v>
       </x:c>
       <x:c r="B26" s="130" t="str">
         <x:v>SA Credit RWA</x:v>
       </x:c>
       <x:c r="C26" s="132" t="n">
-        <x:v>439259.3643725884</x:v>
+        <x:v>438399.64940665517</x:v>
       </x:c>
       <x:c r="D26" s="150" t="b">
         <x:v>0</x:v>
@@ -5990,21 +6145,27 @@
       <x:c r="E26" s="108"/>
       <x:c r="F26" s="108"/>
       <x:c r="G26" s="108"/>
-      <x:c r="H26" s="108"/>
-      <x:c r="I26" s="108"/>
-      <x:c r="J26" s="108"/>
+      <x:c r="H26" s="108" t="str">
+        <x:v>Regulatory retail</x:v>
+      </x:c>
+      <x:c r="I26" s="173" t="n">
+        <x:v>0.7303635271131869</x:v>
+      </x:c>
+      <x:c r="J26" s="173" t="n">
+        <x:v>1.0859747994006865</x:v>
+      </x:c>
       <x:c r="K26" s="108"/>
       <x:c r="L26" s="108"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="130" t="str">
-        <x:v>adverse</x:v>
+        <x:v>Adverse</x:v>
       </x:c>
       <x:c r="B27" s="130" t="str">
         <x:v>IRB Credit RWA</x:v>
       </x:c>
       <x:c r="C27" s="132" t="n">
-        <x:v>976102.9494243957</x:v>
+        <x:v>769539.1397440645</x:v>
       </x:c>
       <x:c r="D27" s="150" t="b">
         <x:v>0</x:v>
@@ -6012,21 +6173,27 @@
       <x:c r="E27" s="108"/>
       <x:c r="F27" s="108"/>
       <x:c r="G27" s="108"/>
-      <x:c r="H27" s="108"/>
-      <x:c r="I27" s="108"/>
-      <x:c r="J27" s="108"/>
+      <x:c r="H27" s="108" t="str">
+        <x:v>Residential RE</x:v>
+      </x:c>
+      <x:c r="I27" s="173" t="n">
+        <x:v>0.33451057228106623</x:v>
+      </x:c>
+      <x:c r="J27" s="173" t="n">
+        <x:v>0.2991358535853657</x:v>
+      </x:c>
       <x:c r="K27" s="108"/>
       <x:c r="L27" s="108"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="130" t="str">
-        <x:v>adverse</x:v>
+        <x:v>Adverse</x:v>
       </x:c>
       <x:c r="B28" s="130" t="str">
-        <x:v>Standardised aggregate RWA base</x:v>
+        <x:v>Standardised Aggregate RWA Base</x:v>
       </x:c>
       <x:c r="C28" s="132" t="n">
-        <x:v>464259.3643725884</x:v>
+        <x:v>463399.64940665517</x:v>
       </x:c>
       <x:c r="D28" s="150" t="b">
         <x:v>0</x:v>
@@ -6034,21 +6201,27 @@
       <x:c r="E28" s="108"/>
       <x:c r="F28" s="108"/>
       <x:c r="G28" s="108"/>
-      <x:c r="H28" s="108"/>
-      <x:c r="I28" s="108"/>
-      <x:c r="J28" s="108"/>
+      <x:c r="H28" s="108" t="str">
+        <x:v>Retail transactor</x:v>
+      </x:c>
+      <x:c r="I28" s="173" t="n">
+        <x:v>0.44046613493181447</x:v>
+      </x:c>
+      <x:c r="J28" s="173" t="n">
+        <x:v>0.8054498005570963</x:v>
+      </x:c>
       <x:c r="K28" s="108"/>
       <x:c r="L28" s="108"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="130" t="str">
-        <x:v>adverse</x:v>
+        <x:v>Adverse</x:v>
       </x:c>
       <x:c r="B29" s="130" t="str">
-        <x:v>Pre-floor model aggregate RWA</x:v>
+        <x:v>Pre-Floor Model Aggregate RWA</x:v>
       </x:c>
       <x:c r="C29" s="132" t="n">
-        <x:v>1001102.9494243957</x:v>
+        <x:v>794539.1397440645</x:v>
       </x:c>
       <x:c r="D29" s="150" t="b">
         <x:v>0</x:v>
@@ -6056,18 +6229,24 @@
       <x:c r="E29" s="108"/>
       <x:c r="F29" s="108"/>
       <x:c r="G29" s="108"/>
-      <x:c r="H29" s="108"/>
-      <x:c r="I29" s="108"/>
-      <x:c r="J29" s="108"/>
+      <x:c r="H29" s="108" t="str">
+        <x:v>Revolving retail</x:v>
+      </x:c>
+      <x:c r="I29" s="173" t="n">
+        <x:v>0.730582505096762</x:v>
+      </x:c>
+      <x:c r="J29" s="173" t="n">
+        <x:v>0.8226483039769329</x:v>
+      </x:c>
       <x:c r="K29" s="108"/>
       <x:c r="L29" s="108"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="130" t="str">
-        <x:v>adverse</x:v>
+        <x:v>Adverse</x:v>
       </x:c>
       <x:c r="B30" s="130" t="str">
-        <x:v>Output-floor rate</x:v>
+        <x:v>Output-Floor Rate</x:v>
       </x:c>
       <x:c r="C30" s="133" t="n">
         <x:v>0.65</x:v>
@@ -6078,21 +6257,27 @@
       <x:c r="E30" s="108"/>
       <x:c r="F30" s="108"/>
       <x:c r="G30" s="108"/>
-      <x:c r="H30" s="108"/>
-      <x:c r="I30" s="108"/>
-      <x:c r="J30" s="108"/>
+      <x:c r="H30" s="108" t="str">
+        <x:v>Sovereign</x:v>
+      </x:c>
+      <x:c r="I30" s="173" t="n">
+        <x:v>0.13646236070442802</x:v>
+      </x:c>
+      <x:c r="J30" s="173" t="n">
+        <x:v>0.18276662735672408</x:v>
+      </x:c>
       <x:c r="K30" s="108"/>
       <x:c r="L30" s="108"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="130" t="str">
-        <x:v>adverse</x:v>
+        <x:v>Adverse</x:v>
       </x:c>
       <x:c r="B31" s="130" t="str">
-        <x:v>Output-floor amount</x:v>
+        <x:v>Output-Floor Amount</x:v>
       </x:c>
       <x:c r="C31" s="132" t="n">
-        <x:v>301768.58684218244</x:v>
+        <x:v>301209.7721143259</x:v>
       </x:c>
       <x:c r="D31" s="150" t="b">
         <x:v>0</x:v>
@@ -6108,13 +6293,13 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="130" t="str">
-        <x:v>adverse</x:v>
+        <x:v>Adverse</x:v>
       </x:c>
       <x:c r="B32" s="130" t="str">
-        <x:v>Final aggregate RWA</x:v>
+        <x:v>Final Aggregate RWA</x:v>
       </x:c>
       <x:c r="C32" s="132" t="n">
-        <x:v>1001102.9494243957</x:v>
+        <x:v>794539.1397440645</x:v>
       </x:c>
       <x:c r="D32" s="150" t="b">
         <x:v>0</x:v>
@@ -6130,10 +6315,10 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="130" t="str">
-        <x:v>adverse</x:v>
+        <x:v>Adverse</x:v>
       </x:c>
       <x:c r="B33" s="130" t="str">
-        <x:v>Floor uplift</x:v>
+        <x:v>Floor Uplift</x:v>
       </x:c>
       <x:c r="C33" s="132" t="n">
         <x:v>0</x:v>
@@ -6152,13 +6337,13 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="130" t="str">
-        <x:v>severe</x:v>
+        <x:v>Severe</x:v>
       </x:c>
       <x:c r="B34" s="130" t="str">
         <x:v>SA Credit RWA</x:v>
       </x:c>
       <x:c r="C34" s="132" t="n">
-        <x:v>484985.19677965663</x:v>
+        <x:v>484304.75527870364</x:v>
       </x:c>
       <x:c r="D34" s="150" t="b">
         <x:v>0</x:v>
@@ -6174,13 +6359,13 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="130" t="str">
-        <x:v>severe</x:v>
+        <x:v>Severe</x:v>
       </x:c>
       <x:c r="B35" s="130" t="str">
         <x:v>IRB Credit RWA</x:v>
       </x:c>
       <x:c r="C35" s="132" t="n">
-        <x:v>1267671.0865599755</x:v>
+        <x:v>988975.0971355619</x:v>
       </x:c>
       <x:c r="D35" s="150" t="b">
         <x:v>0</x:v>
@@ -6196,13 +6381,13 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="130" t="str">
-        <x:v>severe</x:v>
+        <x:v>Severe</x:v>
       </x:c>
       <x:c r="B36" s="130" t="str">
-        <x:v>Standardised aggregate RWA base</x:v>
+        <x:v>Standardised Aggregate RWA Base</x:v>
       </x:c>
       <x:c r="C36" s="132" t="n">
-        <x:v>509985.19677965663</x:v>
+        <x:v>509304.75527870364</x:v>
       </x:c>
       <x:c r="D36" s="150" t="b">
         <x:v>0</x:v>
@@ -6218,13 +6403,13 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="130" t="str">
-        <x:v>severe</x:v>
+        <x:v>Severe</x:v>
       </x:c>
       <x:c r="B37" s="130" t="str">
-        <x:v>Pre-floor model aggregate RWA</x:v>
+        <x:v>Pre-Floor Model Aggregate RWA</x:v>
       </x:c>
       <x:c r="C37" s="132" t="n">
-        <x:v>1292671.0865599755</x:v>
+        <x:v>1013975.0971355619</x:v>
       </x:c>
       <x:c r="D37" s="150" t="b">
         <x:v>0</x:v>
@@ -6240,10 +6425,10 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="130" t="str">
-        <x:v>severe</x:v>
+        <x:v>Severe</x:v>
       </x:c>
       <x:c r="B38" s="130" t="str">
-        <x:v>Output-floor rate</x:v>
+        <x:v>Output-Floor Rate</x:v>
       </x:c>
       <x:c r="C38" s="133" t="n">
         <x:v>0.65</x:v>
@@ -6262,13 +6447,13 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="130" t="str">
-        <x:v>severe</x:v>
+        <x:v>Severe</x:v>
       </x:c>
       <x:c r="B39" s="130" t="str">
-        <x:v>Output-floor amount</x:v>
+        <x:v>Output-Floor Amount</x:v>
       </x:c>
       <x:c r="C39" s="132" t="n">
-        <x:v>331490.3779067768</x:v>
+        <x:v>331048.09093115735</x:v>
       </x:c>
       <x:c r="D39" s="150" t="b">
         <x:v>0</x:v>
@@ -6284,13 +6469,13 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="130" t="str">
-        <x:v>severe</x:v>
+        <x:v>Severe</x:v>
       </x:c>
       <x:c r="B40" s="130" t="str">
-        <x:v>Final aggregate RWA</x:v>
+        <x:v>Final Aggregate RWA</x:v>
       </x:c>
       <x:c r="C40" s="132" t="n">
-        <x:v>1292671.0865599755</x:v>
+        <x:v>1013975.0971355619</x:v>
       </x:c>
       <x:c r="D40" s="150" t="b">
         <x:v>0</x:v>
@@ -6306,10 +6491,10 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="135" t="str">
-        <x:v>severe</x:v>
+        <x:v>Severe</x:v>
       </x:c>
       <x:c r="B41" s="135" t="str">
-        <x:v>Floor uplift</x:v>
+        <x:v>Floor Uplift</x:v>
       </x:c>
       <x:c r="C41" s="137" t="n">
         <x:v>0</x:v>
@@ -6333,10 +6518,10 @@
     <x:mergeCell ref="A16:E16"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f25c08ba71c4413"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69242f51d65145ad"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9e27fab0caa457b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b72047312024a40"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80e442426fdb4a0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc48e1e481064dc2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6439,7 +6624,7 @@
         <x:v>Borrower HHI</x:v>
       </x:c>
       <x:c r="B6" s="128" t="n">
-        <x:v>0.0006787721</x:v>
+        <x:v>0.0006700608</x:v>
       </x:c>
       <x:c r="C6" s="108"/>
       <x:c r="D6" s="108"/>
@@ -6457,7 +6642,7 @@
         <x:v>Sector HHI</x:v>
       </x:c>
       <x:c r="B7" s="133" t="n">
-        <x:v>0.1252798127</x:v>
+        <x:v>0.123869662</x:v>
       </x:c>
       <x:c r="C7" s="108"/>
       <x:c r="D7" s="108"/>
@@ -6475,7 +6660,7 @@
         <x:v>Top 10 borrower share</x:v>
       </x:c>
       <x:c r="B8" s="133" t="n">
-        <x:v>0.0206126831</x:v>
+        <x:v>0.0198045207</x:v>
       </x:c>
       <x:c r="C8" s="108"/>
       <x:c r="D8" s="108"/>
@@ -6493,7 +6678,7 @@
         <x:v>Top 20 borrower share</x:v>
       </x:c>
       <x:c r="B9" s="133" t="n">
-        <x:v>0.0375186998</x:v>
+        <x:v>0.0347362902</x:v>
       </x:c>
       <x:c r="C9" s="108"/>
       <x:c r="D9" s="108"/>
@@ -6511,7 +6696,7 @@
         <x:v>Top 5 sector share</x:v>
       </x:c>
       <x:c r="B10" s="136" t="n">
-        <x:v>0.6356088777</x:v>
+        <x:v>0.6371465728</x:v>
       </x:c>
       <x:c r="C10" s="108"/>
       <x:c r="D10" s="108"/>
@@ -6598,25 +6783,25 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="125" t="str">
-        <x:v>BOR-0009623</x:v>
+        <x:v>BOR-0010536</x:v>
       </x:c>
       <x:c r="B15" s="125" t="str">
-        <x:v>GRP-001924</x:v>
+        <x:v>GRP-0010536</x:v>
       </x:c>
       <x:c r="C15" s="127" t="n">
-        <x:v>1759.3022053719596</x:v>
+        <x:v>1825.5839400635919</x:v>
       </x:c>
       <x:c r="D15" s="127" t="n">
-        <x:v>1749.6494423655213</x:v>
+        <x:v>7146.312713593773</x:v>
       </x:c>
       <x:c r="E15" s="126" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F15" s="128" t="n">
-        <x:v>0.002502963</x:v>
+        <x:v>0.0026052398</x:v>
       </x:c>
       <x:c r="G15" s="128" t="n">
-        <x:v>0.002502963</x:v>
+        <x:v>0.0026052398</x:v>
       </x:c>
       <x:c r="H15" s="108"/>
       <x:c r="I15" s="108"/>
@@ -6626,25 +6811,25 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="130" t="str">
-        <x:v>BOR-0010400</x:v>
+        <x:v>BOR-0028988</x:v>
       </x:c>
       <x:c r="B16" s="130" t="str">
-        <x:v>GRP-002080</x:v>
+        <x:v>GRP-0028988</x:v>
       </x:c>
       <x:c r="C16" s="132" t="n">
-        <x:v>1705.4646184421495</x:v>
+        <x:v>1664.611627286871</x:v>
       </x:c>
       <x:c r="D16" s="132" t="n">
-        <x:v>2038.8727453929664</x:v>
+        <x:v>148.27645850516606</x:v>
       </x:c>
       <x:c r="E16" s="131" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F16" s="133" t="n">
-        <x:v>0.0024263682</x:v>
+        <x:v>0.0023755207</x:v>
       </x:c>
       <x:c r="G16" s="133" t="n">
-        <x:v>0.0049293312</x:v>
+        <x:v>0.0049807606</x:v>
       </x:c>
       <x:c r="H16" s="108"/>
       <x:c r="I16" s="108"/>
@@ -6654,25 +6839,25 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="130" t="str">
-        <x:v>BOR-0010237</x:v>
+        <x:v>BOR-0010562</x:v>
       </x:c>
       <x:c r="B17" s="130" t="str">
-        <x:v>GRP-002047</x:v>
+        <x:v>GRP-0010562</x:v>
       </x:c>
       <x:c r="C17" s="132" t="n">
-        <x:v>1572.3991842653902</x:v>
+        <x:v>1560.162820246262</x:v>
       </x:c>
       <x:c r="D17" s="132" t="n">
-        <x:v>1541.9085751291423</x:v>
+        <x:v>1464.3769196285423</x:v>
       </x:c>
       <x:c r="E17" s="131" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F17" s="133" t="n">
-        <x:v>0.0022370557</x:v>
+        <x:v>0.0022264648</x:v>
       </x:c>
       <x:c r="G17" s="133" t="n">
-        <x:v>0.0071663869</x:v>
+        <x:v>0.0072072253</x:v>
       </x:c>
       <x:c r="H17" s="108"/>
       <x:c r="I17" s="108"/>
@@ -6682,25 +6867,25 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="130" t="str">
-        <x:v>BOR-0009856</x:v>
+        <x:v>BOR-0010365</x:v>
       </x:c>
       <x:c r="B18" s="130" t="str">
-        <x:v>GRP-001971</x:v>
+        <x:v>GRP-0010365</x:v>
       </x:c>
       <x:c r="C18" s="132" t="n">
-        <x:v>1548.8969722621255</x:v>
+        <x:v>1488.5001315838597</x:v>
       </x:c>
       <x:c r="D18" s="132" t="n">
-        <x:v>845.9715407916749</x:v>
+        <x:v>943.5188972539318</x:v>
       </x:c>
       <x:c r="E18" s="131" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F18" s="133" t="n">
-        <x:v>0.002203619</x:v>
+        <x:v>0.0021241969</x:v>
       </x:c>
       <x:c r="G18" s="133" t="n">
-        <x:v>0.0093700059</x:v>
+        <x:v>0.0093314223</x:v>
       </x:c>
       <x:c r="H18" s="108"/>
       <x:c r="I18" s="108"/>
@@ -6710,25 +6895,25 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="130" t="str">
-        <x:v>BOR-0010114</x:v>
+        <x:v>BOR-0028721</x:v>
       </x:c>
       <x:c r="B19" s="130" t="str">
-        <x:v>GRP-002022</x:v>
+        <x:v>GRP-0028721</x:v>
       </x:c>
       <x:c r="C19" s="132" t="n">
-        <x:v>1442.39675901072</x:v>
+        <x:v>1383.0273144935031</x:v>
       </x:c>
       <x:c r="D19" s="132" t="n">
-        <x:v>1104.2990255126115</x:v>
+        <x:v>115.04473247114666</x:v>
       </x:c>
       <x:c r="E19" s="131" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F19" s="133" t="n">
-        <x:v>0.002052101</x:v>
+        <x:v>0.0019736796</x:v>
       </x:c>
       <x:c r="G19" s="133" t="n">
-        <x:v>0.0114221068</x:v>
+        <x:v>0.0113051019</x:v>
       </x:c>
       <x:c r="H19" s="108"/>
       <x:c r="I19" s="108"/>
@@ -6738,25 +6923,25 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="130" t="str">
-        <x:v>BOR-0028723</x:v>
+        <x:v>BOR-0010405</x:v>
       </x:c>
       <x:c r="B20" s="130" t="str">
-        <x:v>GRP-005744</x:v>
+        <x:v>GRP-0010405</x:v>
       </x:c>
       <x:c r="C20" s="132" t="n">
-        <x:v>1349.0300955525483</x:v>
+        <x:v>1268.2170823834867</x:v>
       </x:c>
       <x:c r="D20" s="132" t="n">
-        <x:v>278.10453779027284</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E20" s="131" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F20" s="133" t="n">
-        <x:v>0.001919268</x:v>
+        <x:v>0.0018098372</x:v>
       </x:c>
       <x:c r="G20" s="133" t="n">
-        <x:v>0.0133413748</x:v>
+        <x:v>0.0131149391</x:v>
       </x:c>
       <x:c r="H20" s="108"/>
       <x:c r="I20" s="108"/>
@@ -6766,25 +6951,25 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="130" t="str">
-        <x:v>BOR-0010435</x:v>
+        <x:v>BOR-0010142</x:v>
       </x:c>
       <x:c r="B21" s="130" t="str">
-        <x:v>GRP-002087</x:v>
+        <x:v>GRP-0010142</x:v>
       </x:c>
       <x:c r="C21" s="132" t="n">
-        <x:v>1309.1001570319245</x:v>
+        <x:v>1251.2597998486783</x:v>
       </x:c>
       <x:c r="D21" s="132" t="n">
-        <x:v>6938.381566463965</x:v>
+        <x:v>491.650378078862</x:v>
       </x:c>
       <x:c r="E21" s="131" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F21" s="133" t="n">
-        <x:v>0.0018624596</x:v>
+        <x:v>0.0017856379</x:v>
       </x:c>
       <x:c r="G21" s="133" t="n">
-        <x:v>0.0152038344</x:v>
+        <x:v>0.014900577</x:v>
       </x:c>
       <x:c r="H21" s="108"/>
       <x:c r="I21" s="108"/>
@@ -6794,25 +6979,25 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="130" t="str">
-        <x:v>BOR-0009694</x:v>
+        <x:v>BOR-0010265</x:v>
       </x:c>
       <x:c r="B22" s="130" t="str">
-        <x:v>GRP-001938</x:v>
+        <x:v>GRP-0010265</x:v>
       </x:c>
       <x:c r="C22" s="132" t="n">
-        <x:v>1295.9272565581714</x:v>
+        <x:v>1209.7821143627575</x:v>
       </x:c>
       <x:c r="D22" s="132" t="n">
-        <x:v>1467.4368198469083</x:v>
+        <x:v>559.7824102779567</x:v>
       </x:c>
       <x:c r="E22" s="131" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F22" s="133" t="n">
-        <x:v>0.0018437185</x:v>
+        <x:v>0.0017264462</x:v>
       </x:c>
       <x:c r="G22" s="133" t="n">
-        <x:v>0.0170475529</x:v>
+        <x:v>0.0166270232</x:v>
       </x:c>
       <x:c r="H22" s="108"/>
       <x:c r="I22" s="108"/>
@@ -6822,25 +7007,25 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="130" t="str">
-        <x:v>BOR-0009603</x:v>
+        <x:v>BOR-0009786</x:v>
       </x:c>
       <x:c r="B23" s="130" t="str">
-        <x:v>GRP-001920</x:v>
+        <x:v>GRP-0009786</x:v>
       </x:c>
       <x:c r="C23" s="132" t="n">
-        <x:v>1284.005649839699</x:v>
+        <x:v>1126.1384626058132</x:v>
       </x:c>
       <x:c r="D23" s="132" t="n">
-        <x:v>3751.241907985839</x:v>
+        <x:v>203.31863104395165</x:v>
       </x:c>
       <x:c r="E23" s="131" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F23" s="133" t="n">
-        <x:v>0.0018267576</x:v>
+        <x:v>0.0016070807</x:v>
       </x:c>
       <x:c r="G23" s="133" t="n">
-        <x:v>0.0188743105</x:v>
+        <x:v>0.0182341039</x:v>
       </x:c>
       <x:c r="H23" s="108"/>
       <x:c r="I23" s="108"/>
@@ -6850,25 +7035,25 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="130" t="str">
-        <x:v>BOR-0010389</x:v>
+        <x:v>BOR-0009862</x:v>
       </x:c>
       <x:c r="B24" s="130" t="str">
-        <x:v>GRP-002077</x:v>
+        <x:v>GRP-0009862</x:v>
       </x:c>
       <x:c r="C24" s="132" t="n">
-        <x:v>1221.880911603844</x:v>
+        <x:v>1100.446750551612</x:v>
       </x:c>
       <x:c r="D24" s="132" t="n">
-        <x:v>1523.4970290830458</x:v>
+        <x:v>709.635567109764</x:v>
       </x:c>
       <x:c r="E24" s="131" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F24" s="133" t="n">
-        <x:v>0.0017383726</x:v>
+        <x:v>0.0015704168</x:v>
       </x:c>
       <x:c r="G24" s="133" t="n">
-        <x:v>0.0206126831</x:v>
+        <x:v>0.0198045207</x:v>
       </x:c>
       <x:c r="H24" s="108"/>
       <x:c r="I24" s="108"/>
@@ -6878,25 +7063,25 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="130" t="str">
-        <x:v>BOR-0010551</x:v>
+        <x:v>BOR-0009868</x:v>
       </x:c>
       <x:c r="B25" s="130" t="str">
-        <x:v>GRP-002110</x:v>
+        <x:v>GRP-0009868</x:v>
       </x:c>
       <x:c r="C25" s="132" t="n">
-        <x:v>1207.6741702070638</x:v>
+        <x:v>1096.8247350297374</x:v>
       </x:c>
       <x:c r="D25" s="132" t="n">
-        <x:v>432.7245286987209</x:v>
+        <x:v>553.9615233453375</x:v>
       </x:c>
       <x:c r="E25" s="131" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F25" s="133" t="n">
-        <x:v>0.0017181606</x:v>
+        <x:v>0.0015652479</x:v>
       </x:c>
       <x:c r="G25" s="133" t="n">
-        <x:v>0.0223308437</x:v>
+        <x:v>0.0213697687</x:v>
       </x:c>
       <x:c r="H25" s="108"/>
       <x:c r="I25" s="108"/>
@@ -6906,25 +7091,25 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="130" t="str">
-        <x:v>BOR-0009779</x:v>
+        <x:v>BOR-0010296</x:v>
       </x:c>
       <x:c r="B26" s="130" t="str">
-        <x:v>GRP-001955</x:v>
+        <x:v>GRP-0010296</x:v>
       </x:c>
       <x:c r="C26" s="132" t="n">
-        <x:v>1205.7514913571983</x:v>
+        <x:v>1090.501009828129</x:v>
       </x:c>
       <x:c r="D26" s="132" t="n">
-        <x:v>1227.7703216907148</x:v>
+        <x:v>569.6088503649244</x:v>
       </x:c>
       <x:c r="E26" s="131" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F26" s="133" t="n">
-        <x:v>0.0017154252</x:v>
+        <x:v>0.0015562235</x:v>
       </x:c>
       <x:c r="G26" s="133" t="n">
-        <x:v>0.0240462689</x:v>
+        <x:v>0.0229259922</x:v>
       </x:c>
       <x:c r="H26" s="108"/>
       <x:c r="I26" s="108"/>
@@ -6934,25 +7119,25 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="130" t="str">
-        <x:v>BOR-0010451</x:v>
+        <x:v>BOR-0010028</x:v>
       </x:c>
       <x:c r="B27" s="130" t="str">
-        <x:v>GRP-002090</x:v>
+        <x:v>GRP-0010028</x:v>
       </x:c>
       <x:c r="C27" s="132" t="n">
-        <x:v>1204.6555587187402</x:v>
+        <x:v>1084.176192226911</x:v>
       </x:c>
       <x:c r="D27" s="132" t="n">
-        <x:v>1909.801014421022</x:v>
+        <x:v>1538.212300267653</x:v>
       </x:c>
       <x:c r="E27" s="131" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F27" s="133" t="n">
-        <x:v>0.001713866</x:v>
+        <x:v>0.0015471975</x:v>
       </x:c>
       <x:c r="G27" s="133" t="n">
-        <x:v>0.025760135</x:v>
+        <x:v>0.0244731897</x:v>
       </x:c>
       <x:c r="H27" s="108"/>
       <x:c r="I27" s="108"/>
@@ -6962,25 +7147,25 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="130" t="str">
-        <x:v>BOR-0009915</x:v>
+        <x:v>BOR-0010589</x:v>
       </x:c>
       <x:c r="B28" s="130" t="str">
-        <x:v>GRP-001983</x:v>
+        <x:v>GRP-0010589</x:v>
       </x:c>
       <x:c r="C28" s="132" t="n">
-        <x:v>1199.4026854635933</x:v>
+        <x:v>1052.4966157537788</x:v>
       </x:c>
       <x:c r="D28" s="132" t="n">
-        <x:v>1328.9540507002175</x:v>
+        <x:v>1225.0206134714638</x:v>
       </x:c>
       <x:c r="E28" s="131" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F28" s="133" t="n">
-        <x:v>0.0017063928</x:v>
+        <x:v>0.0015019885</x:v>
       </x:c>
       <x:c r="G28" s="133" t="n">
-        <x:v>0.0274665278</x:v>
+        <x:v>0.0259751782</x:v>
       </x:c>
       <x:c r="H28" s="108"/>
       <x:c r="I28" s="108"/>
@@ -6990,25 +7175,25 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="130" t="str">
-        <x:v>BOR-0010060</x:v>
+        <x:v>BOR-0010584</x:v>
       </x:c>
       <x:c r="B29" s="130" t="str">
-        <x:v>GRP-002012</x:v>
+        <x:v>GRP-0010584</x:v>
       </x:c>
       <x:c r="C29" s="132" t="n">
-        <x:v>1192.9195083929433</x:v>
+        <x:v>1052.0969604353718</x:v>
       </x:c>
       <x:c r="D29" s="132" t="n">
-        <x:v>554.8105723036848</x:v>
+        <x:v>1368.5673909558625</x:v>
       </x:c>
       <x:c r="E29" s="131" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F29" s="133" t="n">
-        <x:v>0.0016971691</x:v>
+        <x:v>0.0015014182</x:v>
       </x:c>
       <x:c r="G29" s="133" t="n">
-        <x:v>0.0291636969</x:v>
+        <x:v>0.0274765964</x:v>
       </x:c>
       <x:c r="H29" s="108"/>
       <x:c r="I29" s="108"/>
@@ -7018,25 +7203,25 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="130" t="str">
-        <x:v>BOR-0010383</x:v>
+        <x:v>BOR-0009938</x:v>
       </x:c>
       <x:c r="B30" s="130" t="str">
-        <x:v>GRP-002076</x:v>
+        <x:v>GRP-0009938</x:v>
       </x:c>
       <x:c r="C30" s="132" t="n">
-        <x:v>1191.153866196569</x:v>
+        <x:v>1043.288601055507</x:v>
       </x:c>
       <x:c r="D30" s="132" t="n">
-        <x:v>526.6536644009869</x:v>
+        <x:v>834.8159995188429</x:v>
       </x:c>
       <x:c r="E30" s="131" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F30" s="133" t="n">
-        <x:v>0.0016946572</x:v>
+        <x:v>0.001488848</x:v>
       </x:c>
       <x:c r="G30" s="133" t="n">
-        <x:v>0.030858354</x:v>
+        <x:v>0.0289654444</x:v>
       </x:c>
       <x:c r="H30" s="108"/>
       <x:c r="I30" s="108"/>
@@ -7046,25 +7231,25 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="130" t="str">
-        <x:v>BOR-0009701</x:v>
+        <x:v>BOR-0010175</x:v>
       </x:c>
       <x:c r="B31" s="130" t="str">
-        <x:v>GRP-001940</x:v>
+        <x:v>GRP-0010175</x:v>
       </x:c>
       <x:c r="C31" s="132" t="n">
-        <x:v>1182.027417746989</x:v>
+        <x:v>1018.7000651482078</x:v>
       </x:c>
       <x:c r="D31" s="132" t="n">
-        <x:v>611.9489686439692</x:v>
+        <x:v>513.873359767369</x:v>
       </x:c>
       <x:c r="E31" s="131" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F31" s="133" t="n">
-        <x:v>0.0016816729</x:v>
+        <x:v>0.0014537584</x:v>
       </x:c>
       <x:c r="G31" s="133" t="n">
-        <x:v>0.032540027</x:v>
+        <x:v>0.0304192028</x:v>
       </x:c>
       <x:c r="H31" s="108"/>
       <x:c r="I31" s="108"/>
@@ -7074,25 +7259,25 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="130" t="str">
-        <x:v>BOR-0010098</x:v>
+        <x:v>BOR-0028752</x:v>
       </x:c>
       <x:c r="B32" s="130" t="str">
-        <x:v>GRP-002019</x:v>
+        <x:v>GRP-0028752</x:v>
       </x:c>
       <x:c r="C32" s="132" t="n">
-        <x:v>1180.741783098835</x:v>
+        <x:v>1012.199806020995</x:v>
       </x:c>
       <x:c r="D32" s="132" t="n">
-        <x:v>924.0925475414631</x:v>
+        <x:v>135.09298823538873</x:v>
       </x:c>
       <x:c r="E32" s="131" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F32" s="133" t="n">
-        <x:v>0.0016798439</x:v>
+        <x:v>0.0014444821</x:v>
       </x:c>
       <x:c r="G32" s="133" t="n">
-        <x:v>0.0342198708</x:v>
+        <x:v>0.0318636849</x:v>
       </x:c>
       <x:c r="H32" s="108"/>
       <x:c r="I32" s="108"/>
@@ -7102,25 +7287,25 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="130" t="str">
-        <x:v>BOR-0009987</x:v>
+        <x:v>BOR-0009774</x:v>
       </x:c>
       <x:c r="B33" s="130" t="str">
-        <x:v>GRP-001997</x:v>
+        <x:v>GRP-0009774</x:v>
       </x:c>
       <x:c r="C33" s="132" t="n">
-        <x:v>1171.61525582416</x:v>
+        <x:v>1011.7325894334734</x:v>
       </x:c>
       <x:c r="D33" s="132" t="n">
-        <x:v>495.17731293848374</x:v>
+        <x:v>1201.2468382079658</x:v>
       </x:c>
       <x:c r="E33" s="131" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F33" s="133" t="n">
-        <x:v>0.0016668595</x:v>
+        <x:v>0.0014438153</x:v>
       </x:c>
       <x:c r="G33" s="133" t="n">
-        <x:v>0.0358867304</x:v>
+        <x:v>0.0333075002</x:v>
       </x:c>
       <x:c r="H33" s="108"/>
       <x:c r="I33" s="108"/>
@@ -7130,25 +7315,25 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="135" t="str">
-        <x:v>BOR-0009784</x:v>
+        <x:v>BOR-0009968</x:v>
       </x:c>
       <x:c r="B34" s="135" t="str">
-        <x:v>GRP-001956</x:v>
+        <x:v>GRP-0009968</x:v>
       </x:c>
       <x:c r="C34" s="137" t="n">
-        <x:v>1147.0914607597174</x:v>
+        <x:v>1001.2038298091419</x:v>
       </x:c>
       <x:c r="D34" s="137" t="n">
-        <x:v>2334.493481988884</x:v>
+        <x:v>2269.371699830069</x:v>
       </x:c>
       <x:c r="E34" s="138" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F34" s="136" t="n">
-        <x:v>0.0016319695</x:v>
+        <x:v>0.00142879</x:v>
       </x:c>
       <x:c r="G34" s="136" t="n">
-        <x:v>0.0375186998</x:v>
+        <x:v>0.0347362902</x:v>
       </x:c>
       <x:c r="H34" s="108"/>
       <x:c r="I34" s="108"/>
@@ -7249,7 +7434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R754a2f3bc241469e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d73d91f9fd94ec1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7334,7 +7519,7 @@
         <x:v>Prior RWA</x:v>
       </x:c>
       <x:c r="B5" s="127" t="n">
-        <x:v>716958.7103084404</x:v>
+        <x:v>567772.7239439853</x:v>
       </x:c>
       <x:c r="C5" s="125" t="str">
         <x:v>total</x:v>
@@ -7354,7 +7539,7 @@
         <x:v>New business</x:v>
       </x:c>
       <x:c r="B6" s="132" t="n">
-        <x:v>21674.6231583682</x:v>
+        <x:v>21339.619275710564</x:v>
       </x:c>
       <x:c r="C6" s="130" t="str">
         <x:v>change</x:v>
@@ -7374,7 +7559,7 @@
         <x:v>Run-off / repayment</x:v>
       </x:c>
       <x:c r="B7" s="132" t="n">
-        <x:v>-8078.646486982144</x:v>
+        <x:v>-8108.456920960321</x:v>
       </x:c>
       <x:c r="C7" s="130" t="str">
         <x:v>change</x:v>
@@ -7394,7 +7579,7 @@
         <x:v>EAD movement</x:v>
       </x:c>
       <x:c r="B8" s="132" t="n">
-        <x:v>-1974.761537821603</x:v>
+        <x:v>-271.9033130035156</x:v>
       </x:c>
       <x:c r="C8" s="130" t="str">
         <x:v>change</x:v>
@@ -7414,7 +7599,7 @@
         <x:v>Rating / PD migration</x:v>
       </x:c>
       <x:c r="B9" s="132" t="n">
-        <x:v>0</x:v>
+        <x:v>25457.38734699492</x:v>
       </x:c>
       <x:c r="C9" s="130" t="str">
         <x:v>change</x:v>
@@ -7434,7 +7619,7 @@
         <x:v>LGD / collateral</x:v>
       </x:c>
       <x:c r="B10" s="132" t="n">
-        <x:v>96.48223983577385</x:v>
+        <x:v>2750.441713050098</x:v>
       </x:c>
       <x:c r="C10" s="130" t="str">
         <x:v>change</x:v>
@@ -7454,7 +7639,7 @@
         <x:v>Maturity</x:v>
       </x:c>
       <x:c r="B11" s="132" t="n">
-        <x:v>0</x:v>
+        <x:v>-25590.579147802735</x:v>
       </x:c>
       <x:c r="C11" s="130" t="str">
         <x:v>change</x:v>
@@ -7471,10 +7656,10 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="130" t="str">
-        <x:v>Residual</x:v>
+        <x:v>Class / eligibility / default</x:v>
       </x:c>
       <x:c r="B12" s="132" t="n">
-        <x:v>-9.765625e-11</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C12" s="130" t="str">
         <x:v>change</x:v>
@@ -7491,13 +7676,13 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="135" t="str">
-        <x:v>Current RWA</x:v>
+        <x:v>Rounding residual</x:v>
       </x:c>
       <x:c r="B13" s="137" t="n">
-        <x:v>728676.4076818405</x:v>
+        <x:v>1.953125e-10</x:v>
       </x:c>
       <x:c r="C13" s="135" t="str">
-        <x:v>total</x:v>
+        <x:v>change</x:v>
       </x:c>
       <x:c r="D13" s="108"/>
       <x:c r="E13" s="108"/>
@@ -7510,9 +7695,15 @@
       <x:c r="L13" s="108"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="108"/>
-      <x:c r="B14" s="140"/>
-      <x:c r="C14" s="108"/>
+      <x:c r="A14" s="108" t="str">
+        <x:v>Current RWA</x:v>
+      </x:c>
+      <x:c r="B14" s="140" t="n">
+        <x:v>583349.2328979744</x:v>
+      </x:c>
+      <x:c r="C14" s="108" t="str">
+        <x:v>total</x:v>
+      </x:c>
       <x:c r="D14" s="108"/>
       <x:c r="E14" s="108"/>
       <x:c r="F14" s="108"/>
@@ -7538,17 +7729,9 @@
       <x:c r="L15" s="108"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="153" t="str">
-        <x:v>Reconciliation difference</x:v>
-      </x:c>
-      <x:c r="B16" s="154" t="n">
-        <x:f>B5+SUM(B6:B12)-B13</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C16" s="153" t="str">
-        <x:f>IF(ABS(B16)&lt;0.0001,"PASS","FAIL")</x:f>
-        <x:v>PASS</x:v>
-      </x:c>
+      <x:c r="A16" s="153"/>
+      <x:c r="B16" s="154"/>
+      <x:c r="C16" s="153"/>
       <x:c r="D16" s="108"/>
       <x:c r="E16" s="108"/>
       <x:c r="F16" s="108"/>
@@ -7560,9 +7743,17 @@
       <x:c r="L16" s="108"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="108"/>
-      <x:c r="B17" s="140"/>
-      <x:c r="C17" s="108"/>
+      <x:c r="A17" s="108" t="str">
+        <x:v>Reconciliation difference</x:v>
+      </x:c>
+      <x:c r="B17" s="140" t="n">
+        <x:f>B5+SUM(B6:B13)-B14</x:f>
+        <x:v>1.1641532182693481e-10</x:v>
+      </x:c>
+      <x:c r="C17" s="108" t="str">
+        <x:f>IF(ABS(B17)&lt;0.0001,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
       <x:c r="D17" s="108"/>
       <x:c r="E17" s="108"/>
       <x:c r="F17" s="108"/>
@@ -7621,9 +7812,9 @@
     <x:mergeCell ref="A2:L2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28be2df8ae164f78"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd93b33d6cc3347ab"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ac8be45a4464783"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf49f137c8054845"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7720,22 +7911,22 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="125" t="str">
-        <x:v>base</x:v>
+        <x:v>Base</x:v>
       </x:c>
       <x:c r="B5" s="127" t="n">
-        <x:v>702887.8163117705</x:v>
+        <x:v>700735.4648341014</x:v>
       </x:c>
       <x:c r="C5" s="127" t="n">
-        <x:v>406207.69049290236</x:v>
+        <x:v>405323.35943071585</x:v>
       </x:c>
       <x:c r="D5" s="127" t="n">
-        <x:v>728676.4076818405</x:v>
+        <x:v>583349.2328979744</x:v>
       </x:c>
       <x:c r="E5" s="127" t="n">
-        <x:v>13235.315584936732</x:v>
+        <x:v>11753.820884425715</x:v>
       </x:c>
       <x:c r="F5" s="127" t="n">
-        <x:v>753676.4076818405</x:v>
+        <x:v>608349.2328979744</x:v>
       </x:c>
       <x:c r="G5" s="149" t="b">
         <x:v>0</x:v>
@@ -7750,28 +7941,28 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="130" t="str">
-        <x:v>adverse</x:v>
+        <x:v>Adverse</x:v>
       </x:c>
       <x:c r="B6" s="132" t="n">
-        <x:v>749123.8559095626</x:v>
+        <x:v>746518.2834362584</x:v>
       </x:c>
       <x:c r="C6" s="132" t="n">
-        <x:v>439259.3643725884</x:v>
+        <x:v>438399.64940665517</x:v>
       </x:c>
       <x:c r="D6" s="132" t="n">
-        <x:v>976102.9494243957</x:v>
+        <x:v>769539.1397440645</x:v>
       </x:c>
       <x:c r="E6" s="132" t="n">
-        <x:v>19594.823366084973</x:v>
+        <x:v>16773.18307234278</x:v>
       </x:c>
       <x:c r="F6" s="132" t="n">
-        <x:v>1001102.9494243957</x:v>
+        <x:v>794539.1397440645</x:v>
       </x:c>
       <x:c r="G6" s="150" t="b">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H6" s="132" t="n">
-        <x:v>8989.486270914751</x:v>
+        <x:v>8958.219401235103</x:v>
       </x:c>
       <x:c r="I6" s="108"/>
       <x:c r="J6" s="108"/>
@@ -7780,28 +7971,28 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="135" t="str">
-        <x:v>severe</x:v>
+        <x:v>Severe</x:v>
       </x:c>
       <x:c r="B7" s="137" t="n">
-        <x:v>813031.0255505507</x:v>
+        <x:v>810207.1969571185</x:v>
       </x:c>
       <x:c r="C7" s="137" t="n">
-        <x:v>484985.19677965663</x:v>
+        <x:v>484304.75527870364</x:v>
       </x:c>
       <x:c r="D7" s="137" t="n">
-        <x:v>1267671.0865599755</x:v>
+        <x:v>988975.0971355619</x:v>
       </x:c>
       <x:c r="E7" s="137" t="n">
-        <x:v>29975.679405568804</x:v>
+        <x:v>24945.246357225224</x:v>
       </x:c>
       <x:c r="F7" s="137" t="n">
-        <x:v>1292671.0865599755</x:v>
+        <x:v>1013975.0971355619</x:v>
       </x:c>
       <x:c r="G7" s="151" t="b">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H7" s="137" t="n">
-        <x:v>24390.930766516518</x:v>
+        <x:v>24306.21590871355</x:v>
       </x:c>
       <x:c r="I7" s="108"/>
       <x:c r="J7" s="108"/>
@@ -7894,19 +8085,19 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="125" t="str">
-        <x:v>Financial Services</x:v>
+        <x:v>Auto Components</x:v>
       </x:c>
       <x:c r="B13" s="127" t="n">
-        <x:v>132649.33399403136</x:v>
+        <x:v>57473.77884345482</x:v>
       </x:c>
       <x:c r="C13" s="127" t="n">
-        <x:v>222275.21342512616</x:v>
+        <x:v>108367.17015109496</x:v>
       </x:c>
       <x:c r="D13" s="127" t="n">
-        <x:v>89625.8794310948</x:v>
+        <x:v>50893.39130764015</x:v>
       </x:c>
       <x:c r="E13" s="128" t="n">
-        <x:v>0.1662834216</x:v>
+        <x:v>0.1254688022</x:v>
       </x:c>
       <x:c r="F13" s="108"/>
       <x:c r="G13" s="108"/>
@@ -7918,19 +8109,19 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="130" t="str">
-        <x:v>Construction</x:v>
+        <x:v>Real Estate</x:v>
       </x:c>
       <x:c r="B14" s="132" t="n">
-        <x:v>76215.77729539698</x:v>
+        <x:v>58473.76140144328</x:v>
       </x:c>
       <x:c r="C14" s="132" t="n">
-        <x:v>144275.43428246168</x:v>
+        <x:v>108095.46170223912</x:v>
       </x:c>
       <x:c r="D14" s="132" t="n">
-        <x:v>68059.65698706468</x:v>
+        <x:v>49621.70030079584</x:v>
       </x:c>
       <x:c r="E14" s="133" t="n">
-        <x:v>0.1262714822</x:v>
+        <x:v>0.1223336692</x:v>
       </x:c>
       <x:c r="F14" s="108"/>
       <x:c r="G14" s="108"/>
@@ -7942,19 +8133,19 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="130" t="str">
-        <x:v>Real Estate</x:v>
+        <x:v>Financial Services</x:v>
       </x:c>
       <x:c r="B15" s="132" t="n">
-        <x:v>72800.36920605261</x:v>
+        <x:v>88125.88688061282</x:v>
       </x:c>
       <x:c r="C15" s="132" t="n">
-        <x:v>136304.34908693275</x:v>
+        <x:v>137137.50013677005</x:v>
       </x:c>
       <x:c r="D15" s="132" t="n">
-        <x:v>63503.97988088015</x:v>
+        <x:v>49011.61325615722</x:v>
       </x:c>
       <x:c r="E15" s="133" t="n">
-        <x:v>0.1178193076</x:v>
+        <x:v>0.1208296057</x:v>
       </x:c>
       <x:c r="F15" s="108"/>
       <x:c r="G15" s="108"/>
@@ -7966,19 +8157,19 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="130" t="str">
-        <x:v>Auto Components</x:v>
+        <x:v>Textiles</x:v>
       </x:c>
       <x:c r="B16" s="132" t="n">
-        <x:v>67220.0481968937</x:v>
+        <x:v>53961.88452084408</x:v>
       </x:c>
       <x:c r="C16" s="132" t="n">
-        <x:v>124674.02004318444</x:v>
+        <x:v>98940.25225183554</x:v>
       </x:c>
       <x:c r="D16" s="132" t="n">
-        <x:v>57453.97184629076</x:v>
+        <x:v>44978.367730991464</x:v>
       </x:c>
       <x:c r="E16" s="133" t="n">
-        <x:v>0.1065946921</x:v>
+        <x:v>0.1108863406</x:v>
       </x:c>
       <x:c r="F16" s="108"/>
       <x:c r="G16" s="108"/>
@@ -7990,19 +8181,19 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="130" t="str">
-        <x:v>Textiles</x:v>
+        <x:v>Consumer</x:v>
       </x:c>
       <x:c r="B17" s="132" t="n">
-        <x:v>67516.38567801227</x:v>
+        <x:v>73791.51077494054</x:v>
       </x:c>
       <x:c r="C17" s="132" t="n">
-        <x:v>124346.2649702784</x:v>
+        <x:v>115536.355031253</x:v>
       </x:c>
       <x:c r="D17" s="132" t="n">
-        <x:v>56829.87929226612</x:v>
+        <x:v>41744.84425631246</x:v>
       </x:c>
       <x:c r="E17" s="133" t="n">
-        <x:v>0.1054368095</x:v>
+        <x:v>0.102914651</x:v>
       </x:c>
       <x:c r="F17" s="108"/>
       <x:c r="G17" s="108"/>
@@ -8017,16 +8208,16 @@
         <x:v>Metals</x:v>
       </x:c>
       <x:c r="B18" s="132" t="n">
-        <x:v>64672.544566003366</x:v>
+        <x:v>56226.87272523917</x:v>
       </x:c>
       <x:c r="C18" s="132" t="n">
-        <x:v>118508.56836647844</x:v>
+        <x:v>96588.10109677126</x:v>
       </x:c>
       <x:c r="D18" s="132" t="n">
-        <x:v>53836.02380047507</x:v>
+        <x:v>40361.228371532095</x:v>
       </x:c>
       <x:c r="E18" s="133" t="n">
-        <x:v>0.0998822918</x:v>
+        <x:v>0.0995035868</x:v>
       </x:c>
       <x:c r="F18" s="108"/>
       <x:c r="G18" s="108"/>
@@ -8041,16 +8232,16 @@
         <x:v>Healthcare</x:v>
       </x:c>
       <x:c r="B19" s="132" t="n">
-        <x:v>73907.18002545215</x:v>
+        <x:v>68681.83827448396</x:v>
       </x:c>
       <x:c r="C19" s="132" t="n">
-        <x:v>119241.64083684556</x:v>
+        <x:v>108919.5570170735</x:v>
       </x:c>
       <x:c r="D19" s="132" t="n">
-        <x:v>45334.46081139341</x:v>
+        <x:v>40237.71874258954</x:v>
       </x:c>
       <x:c r="E19" s="133" t="n">
-        <x:v>0.084109292</x:v>
+        <x:v>0.0991990953</x:v>
       </x:c>
       <x:c r="F19" s="108"/>
       <x:c r="G19" s="108"/>
@@ -8062,19 +8253,19 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="130" t="str">
-        <x:v>Consumer</x:v>
+        <x:v>Construction</x:v>
       </x:c>
       <x:c r="B20" s="132" t="n">
-        <x:v>77413.87259869809</x:v>
+        <x:v>50542.276874128765</x:v>
       </x:c>
       <x:c r="C20" s="132" t="n">
-        <x:v>120912.79118747903</x:v>
+        <x:v>90777.53565876148</x:v>
       </x:c>
       <x:c r="D20" s="132" t="n">
-        <x:v>43498.91858878094</x:v>
+        <x:v>40235.25878463272</x:v>
       </x:c>
       <x:c r="E20" s="133" t="n">
-        <x:v>0.0807037997</x:v>
+        <x:v>0.0991930307</x:v>
       </x:c>
       <x:c r="F20" s="108"/>
       <x:c r="G20" s="108"/>
@@ -8089,16 +8280,16 @@
         <x:v>IT Services</x:v>
       </x:c>
       <x:c r="B21" s="132" t="n">
-        <x:v>65709.94339051725</x:v>
+        <x:v>48747.04568179307</x:v>
       </x:c>
       <x:c r="C21" s="132" t="n">
-        <x:v>106069.90013007249</x:v>
+        <x:v>78247.05809274894</x:v>
       </x:c>
       <x:c r="D21" s="132" t="n">
-        <x:v>40359.95673955524</x:v>
+        <x:v>29500.01241095587</x:v>
       </x:c>
       <x:c r="E21" s="133" t="n">
-        <x:v>0.0748800653</x:v>
+        <x:v>0.0727271484</x:v>
       </x:c>
       <x:c r="F21" s="108"/>
       <x:c r="G21" s="108"/>
@@ -8113,16 +8304,16 @@
         <x:v>Government</x:v>
       </x:c>
       <x:c r="B22" s="132" t="n">
-        <x:v>28665.82682924301</x:v>
+        <x:v>25475.185787076643</x:v>
       </x:c>
       <x:c r="C22" s="132" t="n">
-        <x:v>46324.849246258076</x:v>
+        <x:v>41761.60311356732</x:v>
       </x:c>
       <x:c r="D22" s="132" t="n">
-        <x:v>17659.022417015065</x:v>
+        <x:v>16286.417326490673</x:v>
       </x:c>
       <x:c r="E22" s="133" t="n">
-        <x:v>0.0327628882</x:v>
+        <x:v>0.0401513285</x:v>
       </x:c>
       <x:c r="F22" s="108"/>
       <x:c r="G22" s="108"/>
@@ -8137,16 +8328,16 @@
         <x:v>Households</x:v>
       </x:c>
       <x:c r="B23" s="137" t="n">
-        <x:v>1905.1259015397159</x:v>
+        <x:v>1849.1911339571884</x:v>
       </x:c>
       <x:c r="C23" s="137" t="n">
-        <x:v>4738.054984858311</x:v>
+        <x:v>4604.502883446744</x:v>
       </x:c>
       <x:c r="D23" s="137" t="n">
-        <x:v>2832.9290833185955</x:v>
+        <x:v>2755.3117494895555</x:v>
       </x:c>
       <x:c r="E23" s="136" t="n">
-        <x:v>0.00525595</x:v>
+        <x:v>0.0067927418</x:v>
       </x:c>
       <x:c r="F23" s="108"/>
       <x:c r="G23" s="108"/>
@@ -8402,10 +8593,10 @@
     <x:mergeCell ref="A11:E11"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc10215953e794e11"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R345fb8a974aa4ac6"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R529d1a31659a4533"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcac5838109ea4458"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R657415f94e034153"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80685f58440d470e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8508,7 +8699,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="125" t="str">
-        <x:v>base</x:v>
+        <x:v>Base</x:v>
       </x:c>
       <x:c r="B5" s="125" t="str">
         <x:v>CET1</x:v>
@@ -8517,33 +8708,33 @@
         <x:v>65000</x:v>
       </x:c>
       <x:c r="D5" s="127" t="n">
-        <x:v>753676.4076818405</x:v>
+        <x:v>608349.2328979744</x:v>
       </x:c>
       <x:c r="E5" s="128" t="n">
-        <x:v>0.0862439096</x:v>
+        <x:v>0.1068465225</x:v>
       </x:c>
       <x:c r="F5" s="128" t="n">
         <x:v>0.07</x:v>
       </x:c>
       <x:c r="G5" s="128" t="n">
-        <x:v>0.0162439096</x:v>
+        <x:v>0.0368465225</x:v>
       </x:c>
       <x:c r="H5" s="127" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I5" s="108"/>
       <x:c r="J5" s="156" t="str">
-        <x:v>base</x:v>
+        <x:v>Base</x:v>
       </x:c>
       <x:c r="K5" s="121" t="n">
         <x:f>E5</x:f>
-        <x:v>0.0862439096</x:v>
+        <x:v>0.1068465225</x:v>
       </x:c>
       <x:c r="L5" s="108"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="130" t="str">
-        <x:v>base</x:v>
+        <x:v>Base</x:v>
       </x:c>
       <x:c r="B6" s="130" t="str">
         <x:v>Tier 1</x:v>
@@ -8552,33 +8743,33 @@
         <x:v>71000</x:v>
       </x:c>
       <x:c r="D6" s="132" t="n">
-        <x:v>753676.4076818405</x:v>
+        <x:v>608349.2328979744</x:v>
       </x:c>
       <x:c r="E6" s="133" t="n">
-        <x:v>0.0942048859</x:v>
+        <x:v>0.1167092784</x:v>
       </x:c>
       <x:c r="F6" s="133" t="n">
         <x:v>0.085</x:v>
       </x:c>
       <x:c r="G6" s="133" t="n">
-        <x:v>0.0092048859</x:v>
+        <x:v>0.0317092784</x:v>
       </x:c>
       <x:c r="H6" s="132" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I6" s="108"/>
       <x:c r="J6" s="156" t="str">
-        <x:v>adverse</x:v>
+        <x:v>Adverse</x:v>
       </x:c>
       <x:c r="K6" s="121" t="n">
         <x:f>E8</x:f>
-        <x:v>0.055948805</x:v>
+        <x:v>0.0705336941</x:v>
       </x:c>
       <x:c r="L6" s="108"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="130" t="str">
-        <x:v>base</x:v>
+        <x:v>Base</x:v>
       </x:c>
       <x:c r="B7" s="130" t="str">
         <x:v>Total Capital</x:v>
@@ -8587,54 +8778,54 @@
         <x:v>80000</x:v>
       </x:c>
       <x:c r="D7" s="132" t="n">
-        <x:v>753676.4076818405</x:v>
+        <x:v>608349.2328979744</x:v>
       </x:c>
       <x:c r="E7" s="133" t="n">
-        <x:v>0.1061463503</x:v>
+        <x:v>0.1315034123</x:v>
       </x:c>
       <x:c r="F7" s="133" t="n">
         <x:v>0.105</x:v>
       </x:c>
       <x:c r="G7" s="133" t="n">
-        <x:v>0.0011463503</x:v>
+        <x:v>0.0265034123</x:v>
       </x:c>
       <x:c r="H7" s="132" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="I7" s="108"/>
       <x:c r="J7" s="156" t="str">
-        <x:v>severe</x:v>
+        <x:v>Severe</x:v>
       </x:c>
       <x:c r="K7" s="121" t="n">
         <x:f>E11</x:f>
-        <x:v>0.0314148507</x:v>
+        <x:v>0.0401329226</x:v>
       </x:c>
       <x:c r="L7" s="108"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="130" t="str">
-        <x:v>adverse</x:v>
+        <x:v>Adverse</x:v>
       </x:c>
       <x:c r="B8" s="130" t="str">
         <x:v>CET1</x:v>
       </x:c>
       <x:c r="C8" s="132" t="n">
-        <x:v>56010.51372908525</x:v>
+        <x:v>56041.78059876489</x:v>
       </x:c>
       <x:c r="D8" s="132" t="n">
-        <x:v>1001102.9494243957</x:v>
+        <x:v>794539.1397440645</x:v>
       </x:c>
       <x:c r="E8" s="133" t="n">
-        <x:v>0.055948805</x:v>
+        <x:v>0.0705336941</x:v>
       </x:c>
       <x:c r="F8" s="133" t="n">
         <x:v>0.07</x:v>
       </x:c>
       <x:c r="G8" s="133" t="n">
-        <x:v>-0.014051195</x:v>
+        <x:v>0.0005336941</x:v>
       </x:c>
       <x:c r="H8" s="132" t="n">
-        <x:v>8989.486270914751</x:v>
+        <x:v>8958.219401235103</x:v>
       </x:c>
       <x:c r="I8" s="108"/>
       <x:c r="J8" s="108"/>
@@ -8643,28 +8834,28 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="130" t="str">
-        <x:v>adverse</x:v>
+        <x:v>Adverse</x:v>
       </x:c>
       <x:c r="B9" s="130" t="str">
         <x:v>Tier 1</x:v>
       </x:c>
       <x:c r="C9" s="132" t="n">
-        <x:v>62010.51372908525</x:v>
+        <x:v>62041.78059876489</x:v>
       </x:c>
       <x:c r="D9" s="132" t="n">
-        <x:v>1001102.9494243957</x:v>
+        <x:v>794539.1397440645</x:v>
       </x:c>
       <x:c r="E9" s="133" t="n">
-        <x:v>0.0619421946</x:v>
+        <x:v>0.0780852415</x:v>
       </x:c>
       <x:c r="F9" s="133" t="n">
         <x:v>0.085</x:v>
       </x:c>
       <x:c r="G9" s="133" t="n">
-        <x:v>-0.0230578054</x:v>
+        <x:v>-0.0069147585</x:v>
       </x:c>
       <x:c r="H9" s="132" t="n">
-        <x:v>8989.486270914751</x:v>
+        <x:v>8958.219401235103</x:v>
       </x:c>
       <x:c r="I9" s="108"/>
       <x:c r="J9" s="108"/>
@@ -8673,28 +8864,28 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="130" t="str">
-        <x:v>adverse</x:v>
+        <x:v>Adverse</x:v>
       </x:c>
       <x:c r="B10" s="130" t="str">
         <x:v>Total Capital</x:v>
       </x:c>
       <x:c r="C10" s="132" t="n">
-        <x:v>71010.51372908526</x:v>
+        <x:v>71041.78059876489</x:v>
       </x:c>
       <x:c r="D10" s="132" t="n">
-        <x:v>1001102.9494243957</x:v>
+        <x:v>794539.1397440645</x:v>
       </x:c>
       <x:c r="E10" s="133" t="n">
-        <x:v>0.070932279</x:v>
+        <x:v>0.0894125626</x:v>
       </x:c>
       <x:c r="F10" s="133" t="n">
         <x:v>0.105</x:v>
       </x:c>
       <x:c r="G10" s="133" t="n">
-        <x:v>-0.034067721</x:v>
+        <x:v>-0.0155874374</x:v>
       </x:c>
       <x:c r="H10" s="132" t="n">
-        <x:v>8989.486270914751</x:v>
+        <x:v>8958.219401235103</x:v>
       </x:c>
       <x:c r="I10" s="108"/>
       <x:c r="J10" s="108"/>
@@ -8703,28 +8894,28 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="130" t="str">
-        <x:v>severe</x:v>
+        <x:v>Severe</x:v>
       </x:c>
       <x:c r="B11" s="130" t="str">
         <x:v>CET1</x:v>
       </x:c>
       <x:c r="C11" s="132" t="n">
-        <x:v>40609.06923348348</x:v>
+        <x:v>40693.78409128645</x:v>
       </x:c>
       <x:c r="D11" s="132" t="n">
-        <x:v>1292671.0865599755</x:v>
+        <x:v>1013975.0971355619</x:v>
       </x:c>
       <x:c r="E11" s="133" t="n">
-        <x:v>0.0314148507</x:v>
+        <x:v>0.0401329226</x:v>
       </x:c>
       <x:c r="F11" s="133" t="n">
         <x:v>0.07</x:v>
       </x:c>
       <x:c r="G11" s="133" t="n">
-        <x:v>-0.0385851493</x:v>
+        <x:v>-0.0298670774</x:v>
       </x:c>
       <x:c r="H11" s="132" t="n">
-        <x:v>24390.930766516518</x:v>
+        <x:v>24306.21590871355</x:v>
       </x:c>
       <x:c r="I11" s="108"/>
       <x:c r="J11" s="108"/>
@@ -8733,28 +8924,28 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="130" t="str">
-        <x:v>severe</x:v>
+        <x:v>Severe</x:v>
       </x:c>
       <x:c r="B12" s="130" t="str">
         <x:v>Tier 1</x:v>
       </x:c>
       <x:c r="C12" s="132" t="n">
-        <x:v>46609.06923348348</x:v>
+        <x:v>46693.78409128645</x:v>
       </x:c>
       <x:c r="D12" s="132" t="n">
-        <x:v>1292671.0865599755</x:v>
+        <x:v>1013975.0971355619</x:v>
       </x:c>
       <x:c r="E12" s="133" t="n">
-        <x:v>0.0360564027</x:v>
+        <x:v>0.0460502277</x:v>
       </x:c>
       <x:c r="F12" s="133" t="n">
         <x:v>0.085</x:v>
       </x:c>
       <x:c r="G12" s="133" t="n">
-        <x:v>-0.0489435973</x:v>
+        <x:v>-0.0389497723</x:v>
       </x:c>
       <x:c r="H12" s="132" t="n">
-        <x:v>24390.930766516518</x:v>
+        <x:v>24306.21590871355</x:v>
       </x:c>
       <x:c r="I12" s="108"/>
       <x:c r="J12" s="108"/>
@@ -8763,28 +8954,28 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="135" t="str">
-        <x:v>severe</x:v>
+        <x:v>Severe</x:v>
       </x:c>
       <x:c r="B13" s="135" t="str">
         <x:v>Total Capital</x:v>
       </x:c>
       <x:c r="C13" s="137" t="n">
-        <x:v>55609.06923348348</x:v>
+        <x:v>55693.78409128645</x:v>
       </x:c>
       <x:c r="D13" s="137" t="n">
-        <x:v>1292671.0865599755</x:v>
+        <x:v>1013975.0971355619</x:v>
       </x:c>
       <x:c r="E13" s="136" t="n">
-        <x:v>0.0430187306</x:v>
+        <x:v>0.0549261853</x:v>
       </x:c>
       <x:c r="F13" s="136" t="n">
         <x:v>0.105</x:v>
       </x:c>
       <x:c r="G13" s="136" t="n">
-        <x:v>-0.0619812694</x:v>
+        <x:v>-0.0500738147</x:v>
       </x:c>
       <x:c r="H13" s="137" t="n">
-        <x:v>24390.930766516518</x:v>
+        <x:v>24306.21590871355</x:v>
       </x:c>
       <x:c r="I13" s="108"/>
       <x:c r="J13" s="108"/>
@@ -8903,9 +9094,9 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73bd80c657d54318"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9e30dd1ebe546b1"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4774129fa684a66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91acf86c6f684eb5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>